<commit_message>
Refresh MatchBalance samples after renderer update
</commit_message>
<xml_diff>
--- a/docs/design/matchbalance-excel/director-workbook-sample.xlsx
+++ b/docs/design/matchbalance-excel/director-workbook-sample.xlsx
@@ -12,9 +12,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'U10 Boys'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$K$16</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$K$15</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'U12 Girls'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$K$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$K$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -246,13 +246,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Cohort1" displayName="Cohort1" ref="A6:K12" headerRowCount="1">
   <autoFilter ref="A6:K12"/>
   <tableColumns count="11">
-    <tableColumn id="1" name="Suggested seed"/>
+    <tableColumn id="1" name="MatchBalance seed"/>
     <tableColumn id="2" name="Team name"/>
     <tableColumn id="3" name="Club"/>
-    <tableColumn id="4" name="PitchRank score"/>
+    <tableColumn id="4" name="PowerScore"/>
     <tableColumn id="5" name="State rank"/>
-    <tableColumn id="6" name="Strength marker"/>
-    <tableColumn id="7" name="Placement status"/>
+    <tableColumn id="6" name="PowerScore seed"/>
+    <tableColumn id="7" name="Movement / placement notes"/>
     <tableColumn id="8" name="Final division"/>
     <tableColumn id="9" name="Pool"/>
     <tableColumn id="10" name="Final seed"/>
@@ -266,13 +266,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Cohort2" displayName="Cohort2" ref="A6:K13" headerRowCount="1">
   <autoFilter ref="A6:K13"/>
   <tableColumns count="11">
-    <tableColumn id="1" name="Suggested seed"/>
+    <tableColumn id="1" name="MatchBalance seed"/>
     <tableColumn id="2" name="Team name"/>
     <tableColumn id="3" name="Club"/>
-    <tableColumn id="4" name="PitchRank score"/>
+    <tableColumn id="4" name="PowerScore"/>
     <tableColumn id="5" name="State rank"/>
-    <tableColumn id="6" name="Strength marker"/>
-    <tableColumn id="7" name="Placement status"/>
+    <tableColumn id="6" name="PowerScore seed"/>
+    <tableColumn id="7" name="Movement / placement notes"/>
     <tableColumn id="8" name="Final division"/>
     <tableColumn id="9" name="Pool"/>
     <tableColumn id="10" name="Final seed"/>
@@ -571,16 +571,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
@@ -604,7 +604,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Start with the numbered seed order. Higher PowerScores indicate greater published strength; bars use the same 0–100 scale. Score steps highlight larger differences supported by nearby matchups; they do not assign divisions or pools.</t>
+          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark larger PowerScore steps supported by nearby matchups; they do not assign divisions or pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Suggested seed</t>
+          <t>MatchBalance seed</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -640,7 +640,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>PitchRank score</t>
+          <t>PowerScore</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -650,12 +650,12 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Strength marker</t>
+          <t>PowerScore seed</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Placement status</t>
+          <t>Movement / placement notes</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -701,7 +701,9 @@
           <t>AZ #2</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr"/>
+      <c r="F7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Seeded</t>
@@ -734,7 +736,9 @@
           <t>AZ #6</t>
         </is>
       </c>
-      <c r="F8" s="12" t="inlineStr"/>
+      <c r="F8" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
           <t>Seeded</t>
@@ -767,10 +771,12 @@
           <t>AZ #11</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr"/>
+      <c r="F9" s="6" t="n">
+        <v>3</v>
+      </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Seeded</t>
+          <t>Very close: seeds 1-3 · Seeded</t>
         </is>
       </c>
       <c r="H9" s="9" t="inlineStr"/>
@@ -800,7 +806,9 @@
           <t>AZ #24</t>
         </is>
       </c>
-      <c r="F10" s="12" t="inlineStr"/>
+      <c r="F10" s="11" t="n">
+        <v>4</v>
+      </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
           <t>Seeded</t>
@@ -833,10 +841,12 @@
           <t>AZ #32</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr"/>
+      <c r="F11" s="6" t="n">
+        <v>5</v>
+      </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Seeded</t>
+          <t>Very close: seeds 4-5 · Seeded</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr"/>
@@ -858,7 +868,7 @@
       </c>
       <c r="D12" s="11" t="n"/>
       <c r="E12" s="11" t="inlineStr"/>
-      <c r="F12" s="12" t="inlineStr"/>
+      <c r="F12" s="11" t="n"/>
       <c r="G12" s="12" t="inlineStr">
         <is>
           <t>Not found in PitchRank</t>
@@ -879,24 +889,16 @@
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="14" t="inlineStr">
         <is>
-          <t>Seed 3 is 11.7 points above seed 4.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
           <t>Sample workbook: use the yellow columns for the director's final decisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="6">
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A15:K15"/>
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A16:K16"/>
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A1:K1"/>
   </mergeCells>
@@ -931,16 +933,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
@@ -964,7 +966,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Start with the numbered seed order. Higher PowerScores indicate greater published strength; bars use the same 0–100 scale. Score steps highlight larger differences supported by nearby matchups; they do not assign divisions or pools.</t>
+          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark larger PowerScore steps supported by nearby matchups; they do not assign divisions or pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
         </is>
       </c>
     </row>
@@ -985,7 +987,7 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Suggested seed</t>
+          <t>MatchBalance seed</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -1000,7 +1002,7 @@
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>PitchRank score</t>
+          <t>PowerScore</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -1010,12 +1012,12 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Strength marker</t>
+          <t>PowerScore seed</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Placement status</t>
+          <t>Movement / placement notes</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -1061,7 +1063,9 @@
           <t>CO #4</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr"/>
+      <c r="F7" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Seeded</t>
@@ -1094,7 +1098,9 @@
           <t>CO #9</t>
         </is>
       </c>
-      <c r="F8" s="12" t="inlineStr"/>
+      <c r="F8" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
           <t>Seeded</t>
@@ -1105,7 +1111,7 @@
       <c r="J8" s="10" t="inlineStr"/>
       <c r="K8" s="9" t="inlineStr"/>
     </row>
-    <row r="9" ht="45" customHeight="1">
+    <row r="9" ht="60" customHeight="1">
       <c r="A9" s="15" t="n">
         <v>3</v>
       </c>
@@ -1127,14 +1133,12 @@
           <t>CO #15</t>
         </is>
       </c>
-      <c r="F9" s="16" t="inlineStr">
-        <is>
-          <t>Score step: 12.3 points between seeds 3 and 4.</t>
-        </is>
+      <c r="F9" s="15" t="n">
+        <v>3</v>
       </c>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>Seeded</t>
+          <t>Competitive Break: 12.3 PowerScore points between seeds 3 and 4. · Very close: seeds 1-3 · Seeded</t>
         </is>
       </c>
       <c r="H9" s="18" t="inlineStr"/>
@@ -1164,7 +1168,9 @@
           <t>CO #29</t>
         </is>
       </c>
-      <c r="F10" s="12" t="inlineStr"/>
+      <c r="F10" s="11" t="n">
+        <v>4</v>
+      </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
           <t>Seeded</t>
@@ -1198,7 +1204,9 @@
           <t>CO #37</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr"/>
+      <c r="F11" s="6" t="n">
+        <v>5</v>
+      </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Seeded</t>
@@ -1231,10 +1239,12 @@
           <t>CO #42</t>
         </is>
       </c>
-      <c r="F12" s="12" t="inlineStr"/>
+      <c r="F12" s="11" t="n">
+        <v>6</v>
+      </c>
       <c r="G12" s="12" t="inlineStr">
         <is>
-          <t>Seeded</t>
+          <t>Very close: seeds 4-6 · Seeded</t>
         </is>
       </c>
       <c r="H12" s="9" t="inlineStr"/>
@@ -1262,7 +1272,7 @@
           <t>CO #50</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr"/>
+      <c r="F13" s="6" t="n"/>
       <c r="G13" s="7" t="inlineStr">
         <is>
           <t>Data review required</t>
@@ -1283,26 +1293,18 @@
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>Score step: 12.3 points between seeds 3 and 4.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="14" t="inlineStr">
-        <is>
           <t>Sample data only. Strength markers are observations, not automatic divisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="6">
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A16:K16"/>
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A17:K17"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D12">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
Fix MatchBalance competitive boundary analysis
</commit_message>
<xml_diff>
--- a/docs/design/matchbalance-excel/director-workbook-sample.xlsx
+++ b/docs/design/matchbalance-excel/director-workbook-sample.xlsx
@@ -148,23 +148,23 @@
     <xf numFmtId="164" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -604,7 +604,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark larger PowerScore steps supported by nearby matchups; they do not assign divisions or pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
+          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark boundaries where nearby projected matchups meaningfully worsen; the PowerScore difference is supporting context; they do not assign divisions or pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
         </is>
       </c>
     </row>
@@ -749,40 +749,40 @@
       <c r="J8" s="10" t="inlineStr"/>
       <c r="K8" s="9" t="inlineStr"/>
     </row>
-    <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="6" t="n">
+    <row r="9" ht="75" customHeight="1">
+      <c r="A9" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>Desert United 2016</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>Desert United</t>
         </is>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="16" t="n">
         <v>84.59999999999999</v>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>AZ #11</t>
         </is>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="F9" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>Very close: seeds 1-3 · Seeded</t>
-        </is>
-      </c>
-      <c r="H9" s="9" t="inlineStr"/>
-      <c r="I9" s="9" t="inlineStr"/>
-      <c r="J9" s="10" t="inlineStr"/>
-      <c r="K9" s="9" t="inlineStr"/>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>Competitive Break: projected matchup quality worsens between seeds 3 and 4; PowerScore difference 11.7 points. · Very close: seeds 1-3 · Seeded</t>
+        </is>
+      </c>
+      <c r="H9" s="17" t="inlineStr"/>
+      <c r="I9" s="17" t="inlineStr"/>
+      <c r="J9" s="18" t="inlineStr"/>
+      <c r="K9" s="17" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="11" t="n">
@@ -887,7 +887,7 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>Sample workbook: use the yellow columns for the director's final decisions.</t>
         </is>
@@ -966,7 +966,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark larger PowerScore steps supported by nearby matchups; they do not assign divisions or pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
+          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark boundaries where nearby projected matchups meaningfully worsen; the PowerScore difference is supporting context; they do not assign divisions or pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
         </is>
       </c>
     </row>
@@ -1111,40 +1111,40 @@
       <c r="J8" s="10" t="inlineStr"/>
       <c r="K8" s="9" t="inlineStr"/>
     </row>
-    <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="15" t="n">
+    <row r="9" ht="75" customHeight="1">
+      <c r="A9" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>Aspen Athletic 2014</t>
         </is>
       </c>
-      <c r="C9" s="16" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>Aspen Athletic</t>
         </is>
       </c>
-      <c r="D9" s="17" t="n">
+      <c r="D9" s="16" t="n">
         <v>83.89999999999999</v>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>CO #15</t>
         </is>
       </c>
-      <c r="F9" s="15" t="n">
+      <c r="F9" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="G9" s="16" t="inlineStr">
-        <is>
-          <t>Competitive Break: 12.3 PowerScore points between seeds 3 and 4. · Very close: seeds 1-3 · Seeded</t>
-        </is>
-      </c>
-      <c r="H9" s="18" t="inlineStr"/>
-      <c r="I9" s="18" t="inlineStr"/>
-      <c r="J9" s="19" t="inlineStr"/>
-      <c r="K9" s="18" t="inlineStr"/>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>Competitive Break: projected matchup quality worsens between seeds 3 and 4; PowerScore difference 12.3 points. · Very close: seeds 1-3 · Seeded</t>
+        </is>
+      </c>
+      <c r="H9" s="17" t="inlineStr"/>
+      <c r="I9" s="17" t="inlineStr"/>
+      <c r="J9" s="18" t="inlineStr"/>
+      <c r="K9" s="17" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="11" t="n">
@@ -1291,7 +1291,7 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Sample data only. Strength markers are observations, not automatic divisions.</t>
         </is>

</xml_diff>

<commit_message>
Add MatchBalance boundary and automatic flight analysis (#1233)
* Fix MatchBalance competitive boundary analysis

* Add complete MatchBalance group assessment

* Add complete MatchBalance flight-plan assessment

* Add automatic MatchBalance flight suggestions

* Fix MatchBalance diagnostic edge cases

* Address MatchBalance review coverage

* Make MatchBalance report squash-safe
</commit_message>
<xml_diff>
--- a/docs/design/matchbalance-excel/director-workbook-sample.xlsx
+++ b/docs/design/matchbalance-excel/director-workbook-sample.xlsx
@@ -148,23 +148,23 @@
     <xf numFmtId="164" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -604,7 +604,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark larger PowerScore steps supported by nearby matchups; they do not assign divisions or pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
+          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark boundaries where nearby projected matchups meaningfully worsen; the PowerScore difference is supporting context; they do not assign divisions or pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
         </is>
       </c>
     </row>
@@ -749,40 +749,40 @@
       <c r="J8" s="10" t="inlineStr"/>
       <c r="K8" s="9" t="inlineStr"/>
     </row>
-    <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="6" t="n">
+    <row r="9" ht="75" customHeight="1">
+      <c r="A9" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>Desert United 2016</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>Desert United</t>
         </is>
       </c>
-      <c r="D9" s="8" t="n">
+      <c r="D9" s="16" t="n">
         <v>84.59999999999999</v>
       </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>AZ #11</t>
         </is>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="F9" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="G9" s="7" t="inlineStr">
-        <is>
-          <t>Very close: seeds 1-3 · Seeded</t>
-        </is>
-      </c>
-      <c r="H9" s="9" t="inlineStr"/>
-      <c r="I9" s="9" t="inlineStr"/>
-      <c r="J9" s="10" t="inlineStr"/>
-      <c r="K9" s="9" t="inlineStr"/>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>Competitive Break: projected matchup quality worsens between seeds 3 and 4; PowerScore difference 11.7 points. · Very close: seeds 1-3 · Seeded</t>
+        </is>
+      </c>
+      <c r="H9" s="17" t="inlineStr"/>
+      <c r="I9" s="17" t="inlineStr"/>
+      <c r="J9" s="18" t="inlineStr"/>
+      <c r="K9" s="17" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="11" t="n">
@@ -887,7 +887,7 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="19" t="inlineStr">
         <is>
           <t>Sample workbook: use the yellow columns for the director's final decisions.</t>
         </is>
@@ -966,7 +966,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark larger PowerScore steps supported by nearby matchups; they do not assign divisions or pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
+          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark boundaries where nearby projected matchups meaningfully worsen; the PowerScore difference is supporting context; they do not assign divisions or pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
         </is>
       </c>
     </row>
@@ -1111,40 +1111,40 @@
       <c r="J8" s="10" t="inlineStr"/>
       <c r="K8" s="9" t="inlineStr"/>
     </row>
-    <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="15" t="n">
+    <row r="9" ht="75" customHeight="1">
+      <c r="A9" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>Aspen Athletic 2014</t>
         </is>
       </c>
-      <c r="C9" s="16" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>Aspen Athletic</t>
         </is>
       </c>
-      <c r="D9" s="17" t="n">
+      <c r="D9" s="16" t="n">
         <v>83.89999999999999</v>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>CO #15</t>
         </is>
       </c>
-      <c r="F9" s="15" t="n">
+      <c r="F9" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="G9" s="16" t="inlineStr">
-        <is>
-          <t>Competitive Break: 12.3 PowerScore points between seeds 3 and 4. · Very close: seeds 1-3 · Seeded</t>
-        </is>
-      </c>
-      <c r="H9" s="18" t="inlineStr"/>
-      <c r="I9" s="18" t="inlineStr"/>
-      <c r="J9" s="19" t="inlineStr"/>
-      <c r="K9" s="18" t="inlineStr"/>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>Competitive Break: projected matchup quality worsens between seeds 3 and 4; PowerScore difference 12.3 points. · Very close: seeds 1-3 · Seeded</t>
+        </is>
+      </c>
+      <c r="H9" s="17" t="inlineStr"/>
+      <c r="I9" s="17" t="inlineStr"/>
+      <c r="J9" s="18" t="inlineStr"/>
+      <c r="K9" s="17" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="11" t="n">
@@ -1291,7 +1291,7 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Sample data only. Strength markers are observations, not automatic divisions.</t>
         </is>

</xml_diff>

<commit_message>
Add practical strength-tier cheat sheets to MatchBalance
</commit_message>
<xml_diff>
--- a/docs/design/matchbalance-excel/director-workbook-sample.xlsx
+++ b/docs/design/matchbalance-excel/director-workbook-sample.xlsx
@@ -12,9 +12,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'U10 Boys'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$K$15</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$K$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'U12 Girls'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$K$16</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$K$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -111,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -121,6 +121,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -571,7 +574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -604,7 +607,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark boundaries where nearby projected matchups meaningfully worsen; the PowerScore difference is supporting context; they do not assign divisions or pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
+          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark boundaries where nearby projected matchups meaningfully worsen; the PowerScore difference is supporting context; they do not assign divisions or pools. Recommended tier breaks use practical division sizes and all potential matchups. A tier can contain multiple pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
         </is>
       </c>
     </row>
@@ -615,269 +618,269 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Seeded: 5 · Not found in PitchRank: 1 · No current rating: 0 · Data review required: 0</t>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Review-required compromise: 5 teams. Seeded: 5 · Not found in PitchRank: 1 · No current rating: 0 · Data review required: 0</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>MatchBalance seed</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Team name</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Club</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>PowerScore</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>State rank</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>PowerScore seed</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Movement / placement notes</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>Final division</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>Pool</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>Final seed</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>Director notes</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Juniper FC 2016 Blue</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Juniper FC</t>
         </is>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="9" t="n">
         <v>90.10000000000001</v>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>AZ #2</t>
         </is>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F7" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>Seeded</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="inlineStr"/>
-      <c r="I7" s="9" t="inlineStr"/>
-      <c r="J7" s="10" t="inlineStr"/>
-      <c r="K7" s="9" t="inlineStr"/>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Tier 1 · Seeded</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr"/>
+      <c r="I7" s="10" t="inlineStr"/>
+      <c r="J7" s="11" t="inlineStr"/>
+      <c r="K7" s="10" t="inlineStr"/>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="11" t="n">
+      <c r="A8" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Copper State 2016</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>Copper State</t>
         </is>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="14" t="n">
         <v>87.2</v>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>AZ #6</t>
         </is>
       </c>
-      <c r="F8" s="11" t="n">
+      <c r="F8" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="G8" s="12" t="inlineStr">
-        <is>
-          <t>Seeded</t>
-        </is>
-      </c>
-      <c r="H8" s="9" t="inlineStr"/>
-      <c r="I8" s="9" t="inlineStr"/>
-      <c r="J8" s="10" t="inlineStr"/>
-      <c r="K8" s="9" t="inlineStr"/>
-    </row>
-    <row r="9" ht="75" customHeight="1">
-      <c r="A9" s="14" t="n">
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>Tier 1 · Seeded</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr"/>
+      <c r="I8" s="10" t="inlineStr"/>
+      <c r="J8" s="11" t="inlineStr"/>
+      <c r="K8" s="10" t="inlineStr"/>
+    </row>
+    <row r="9" ht="105" customHeight="1">
+      <c r="A9" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>Desert United 2016</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>Desert United</t>
         </is>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D9" s="17" t="n">
         <v>84.59999999999999</v>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>AZ #11</t>
         </is>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="F9" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="G9" s="15" t="inlineStr">
-        <is>
-          <t>Competitive Break: projected matchup quality worsens between seeds 3 and 4; PowerScore difference 11.7 points. · Very close: seeds 1-3 · Seeded</t>
-        </is>
-      </c>
-      <c r="H9" s="17" t="inlineStr"/>
-      <c r="I9" s="17" t="inlineStr"/>
-      <c r="J9" s="18" t="inlineStr"/>
-      <c r="K9" s="17" t="inlineStr"/>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Tier 1 · Competitive Break: projected matchup quality worsens between seeds 3 and 4; PowerScore difference 11.7 points. · Competitive Break: natural strength separation · Very close: seeds 1-3 · Seeded</t>
+        </is>
+      </c>
+      <c r="H9" s="18" t="inlineStr"/>
+      <c r="I9" s="18" t="inlineStr"/>
+      <c r="J9" s="19" t="inlineStr"/>
+      <c r="K9" s="18" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="11" t="n">
+      <c r="A10" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Valley Athletic 2016</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>Valley Athletic</t>
         </is>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="14" t="n">
         <v>72.89999999999999</v>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>AZ #24</t>
         </is>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="G10" s="12" t="inlineStr">
-        <is>
-          <t>Seeded</t>
-        </is>
-      </c>
-      <c r="H10" s="9" t="inlineStr"/>
-      <c r="I10" s="9" t="inlineStr"/>
-      <c r="J10" s="10" t="inlineStr"/>
-      <c r="K10" s="9" t="inlineStr"/>
-    </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="6" t="n">
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>Tier 1 · Seeded</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr"/>
+      <c r="I10" s="10" t="inlineStr"/>
+      <c r="J10" s="11" t="inlineStr"/>
+      <c r="K10" s="10" t="inlineStr"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Mesa Juniors 2016</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Mesa Juniors</t>
         </is>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="9" t="n">
         <v>70.09999999999999</v>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>AZ #32</t>
         </is>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>Very close: seeds 4-5 · Seeded</t>
-        </is>
-      </c>
-      <c r="H11" s="9" t="inlineStr"/>
-      <c r="I11" s="9" t="inlineStr"/>
-      <c r="J11" s="10" t="inlineStr"/>
-      <c r="K11" s="9" t="inlineStr"/>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Tier 1 · Very close: seeds 4-5 · Seeded</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr"/>
+      <c r="I11" s="10" t="inlineStr"/>
+      <c r="J11" s="11" t="inlineStr"/>
+      <c r="K11" s="10" t="inlineStr"/>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="11" t="n"/>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Sample Academy 2016</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>Sample Academy</t>
         </is>
       </c>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="inlineStr"/>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="12" t="inlineStr">
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="12" t="inlineStr"/>
+      <c r="F12" s="12" t="n"/>
+      <c r="G12" s="13" t="inlineStr">
         <is>
           <t>Not found in PitchRank</t>
         </is>
       </c>
-      <c r="H12" s="9" t="inlineStr"/>
-      <c r="I12" s="9" t="inlineStr"/>
-      <c r="J12" s="10" t="inlineStr"/>
-      <c r="K12" s="9" t="inlineStr"/>
+      <c r="H12" s="10" t="inlineStr"/>
+      <c r="I12" s="10" t="inlineStr"/>
+      <c r="J12" s="11" t="inlineStr"/>
+      <c r="K12" s="10" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -886,21 +889,61 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="19" t="inlineStr">
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Review-required compromise: Tier 1: seeds 1-5 (5 teams; compatible pools 5; minimum 4 games). Pool memberships remain the director's decision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>5 of 6 teams assessed in the tier order; 1 still need placement. These breaks cover the assessed subset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>Review-required compromise: every evaluated arrangement retains projected mismatches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>Worst remaining mismatch: Juniper FC 2016 Blue vs Mesa Juniors 2016; expected absolute goal difference 4.00, four-goal margin probability 55%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>Formats use the saved MatchBalance profile; confirm game guarantees and event logistics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="20" t="inlineStr">
         <is>
           <t>Sample workbook: use the yellow columns for the director's final decisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="11">
+    <mergeCell ref="A18:K18"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A20:K20"/>
     <mergeCell ref="A15:K15"/>
     <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A16:K16"/>
+    <mergeCell ref="A19:K19"/>
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A17:K17"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D11">
     <cfRule type="dataBar" priority="1">
@@ -933,7 +976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -966,7 +1009,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark boundaries where nearby projected matchups meaningfully worsen; the PowerScore difference is supporting context; they do not assign divisions or pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
+          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark boundaries where nearby projected matchups meaningfully worsen; the PowerScore difference is supporting context; they do not assign divisions or pools. Recommended tier breaks use practical division sizes and all potential matchups. A tier can contain multiple pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
         </is>
       </c>
     </row>
@@ -977,311 +1020,311 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Seeded: 6 · Not found in PitchRank: 0 · No current rating: 0 · Data review required: 1</t>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Suggested tiers: 3 + 3 teams. Seeded: 6 · Not found in PitchRank: 0 · No current rating: 0 · Data review required: 1</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>MatchBalance seed</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Team name</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Club</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>PowerScore</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>State rank</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>PowerScore seed</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Movement / placement notes</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>Final division</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>Pool</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>Final seed</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>Director notes</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Summit SC 2014 Green</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Summit SC</t>
         </is>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="9" t="n">
         <v>89.3</v>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>CO #4</t>
         </is>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F7" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>Seeded</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="inlineStr"/>
-      <c r="I7" s="9" t="inlineStr"/>
-      <c r="J7" s="10" t="inlineStr"/>
-      <c r="K7" s="9" t="inlineStr"/>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Tier 1 · Seeded</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr"/>
+      <c r="I7" s="10" t="inlineStr"/>
+      <c r="J7" s="11" t="inlineStr"/>
+      <c r="K7" s="10" t="inlineStr"/>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="11" t="n">
+      <c r="A8" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Front Range FC 2014</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>Front Range FC</t>
         </is>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="14" t="n">
         <v>86.5</v>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>CO #9</t>
         </is>
       </c>
-      <c r="F8" s="11" t="n">
+      <c r="F8" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="G8" s="12" t="inlineStr">
-        <is>
-          <t>Seeded</t>
-        </is>
-      </c>
-      <c r="H8" s="9" t="inlineStr"/>
-      <c r="I8" s="9" t="inlineStr"/>
-      <c r="J8" s="10" t="inlineStr"/>
-      <c r="K8" s="9" t="inlineStr"/>
-    </row>
-    <row r="9" ht="75" customHeight="1">
-      <c r="A9" s="14" t="n">
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>Tier 1 · Seeded</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr"/>
+      <c r="I8" s="10" t="inlineStr"/>
+      <c r="J8" s="11" t="inlineStr"/>
+      <c r="K8" s="10" t="inlineStr"/>
+    </row>
+    <row r="9" ht="105" customHeight="1">
+      <c r="A9" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>Aspen Athletic 2014</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>Aspen Athletic</t>
         </is>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D9" s="17" t="n">
         <v>83.89999999999999</v>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>CO #15</t>
         </is>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="F9" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="G9" s="15" t="inlineStr">
-        <is>
-          <t>Competitive Break: projected matchup quality worsens between seeds 3 and 4; PowerScore difference 12.3 points. · Very close: seeds 1-3 · Seeded</t>
-        </is>
-      </c>
-      <c r="H9" s="17" t="inlineStr"/>
-      <c r="I9" s="17" t="inlineStr"/>
-      <c r="J9" s="18" t="inlineStr"/>
-      <c r="K9" s="17" t="inlineStr"/>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Tier 1 · Competitive Break: projected matchup quality worsens between seeds 3 and 4; PowerScore difference 12.3 points. · Recommended tier break + natural strength separation · Very close: seeds 1-3 · Seeded</t>
+        </is>
+      </c>
+      <c r="H9" s="18" t="inlineStr"/>
+      <c r="I9" s="18" t="inlineStr"/>
+      <c r="J9" s="19" t="inlineStr"/>
+      <c r="K9" s="18" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="11" t="n">
+      <c r="A10" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Peak United 2014</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>Peak United</t>
         </is>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="14" t="n">
         <v>71.59999999999999</v>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>CO #29</t>
         </is>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="G10" s="12" t="inlineStr">
-        <is>
-          <t>Seeded</t>
-        </is>
-      </c>
-      <c r="H10" s="9" t="inlineStr"/>
-      <c r="I10" s="9" t="inlineStr"/>
-      <c r="J10" s="10" t="inlineStr"/>
-      <c r="K10" s="9" t="inlineStr"/>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 · Seeded</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr"/>
+      <c r="I10" s="10" t="inlineStr"/>
+      <c r="J10" s="11" t="inlineStr"/>
+      <c r="K10" s="10" t="inlineStr"/>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="6" t="n">
+      <c r="A11" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Foothills FC 2014
 Listed: Premier</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Foothills FC</t>
         </is>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="9" t="n">
         <v>68.89999999999999</v>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>CO #37</t>
         </is>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>Seeded</t>
-        </is>
-      </c>
-      <c r="H11" s="9" t="inlineStr"/>
-      <c r="I11" s="9" t="inlineStr"/>
-      <c r="J11" s="10" t="inlineStr"/>
-      <c r="K11" s="9" t="inlineStr"/>
-    </row>
-    <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="11" t="n">
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Tier 2 · Seeded</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr"/>
+      <c r="I11" s="10" t="inlineStr"/>
+      <c r="J11" s="11" t="inlineStr"/>
+      <c r="K11" s="10" t="inlineStr"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Sample Select 2014</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>Sample Select</t>
         </is>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="14" t="n">
         <v>67.40000000000001</v>
       </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="E12" s="12" t="inlineStr">
         <is>
           <t>CO #42</t>
         </is>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="F12" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="G12" s="12" t="inlineStr">
-        <is>
-          <t>Very close: seeds 4-6 · Seeded</t>
-        </is>
-      </c>
-      <c r="H12" s="9" t="inlineStr"/>
-      <c r="I12" s="9" t="inlineStr"/>
-      <c r="J12" s="10" t="inlineStr"/>
-      <c r="K12" s="9" t="inlineStr"/>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 · Very close: seeds 4-6 · Seeded</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr"/>
+      <c r="I12" s="10" t="inlineStr"/>
+      <c r="J12" s="11" t="inlineStr"/>
+      <c r="K12" s="10" t="inlineStr"/>
     </row>
     <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="6" t="n"/>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="A13" s="7" t="n"/>
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Review United 2014</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Review United</t>
         </is>
       </c>
-      <c r="D13" s="8" t="n">
+      <c r="D13" s="9" t="n">
         <v>65</v>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>CO #50</t>
         </is>
       </c>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="8" t="inlineStr">
         <is>
           <t>Data review required</t>
         </is>
       </c>
-      <c r="H13" s="9" t="inlineStr"/>
-      <c r="I13" s="9" t="inlineStr"/>
-      <c r="J13" s="10" t="inlineStr"/>
-      <c r="K13" s="9" t="inlineStr"/>
+      <c r="H13" s="10" t="inlineStr"/>
+      <c r="I13" s="10" t="inlineStr"/>
+      <c r="J13" s="11" t="inlineStr"/>
+      <c r="K13" s="10" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1290,21 +1333,45 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="19" t="inlineStr">
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>Suggested tiers: Tier 1: seeds 1-3 (3 teams; compatible pools 3; minimum 2 games); Tier 2: seeds 4-6 (3 teams; compatible pools 3; minimum 2 games). Pool memberships remain the director's decision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>6 of 7 teams assessed in the tier order; 1 still need placement. These breaks cover the assessed subset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>Formats use the saved MatchBalance profile; confirm game guarantees and event logistics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>Sample data only. Strength markers are observations, not automatic divisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="9">
+    <mergeCell ref="A18:K18"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A16:K16"/>
+    <mergeCell ref="A19:K19"/>
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A17:K17"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D12">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
Add practical strength-tier cheat sheets to MatchBalance (#1262)
</commit_message>
<xml_diff>
--- a/docs/design/matchbalance-excel/director-workbook-sample.xlsx
+++ b/docs/design/matchbalance-excel/director-workbook-sample.xlsx
@@ -12,9 +12,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'U10 Boys'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$K$15</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$K$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'U12 Girls'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$K$16</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$K$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -111,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -121,6 +121,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -571,7 +574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -604,7 +607,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark boundaries where nearby projected matchups meaningfully worsen; the PowerScore difference is supporting context; they do not assign divisions or pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
+          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark boundaries where nearby projected matchups meaningfully worsen; the PowerScore difference is supporting context; they do not assign divisions or pools. Recommended tier breaks use practical division sizes and all potential matchups. A tier can contain multiple pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
         </is>
       </c>
     </row>
@@ -615,269 +618,269 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Seeded: 5 · Not found in PitchRank: 1 · No current rating: 0 · Data review required: 0</t>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Review-required compromise: 5 teams. Seeded: 5 · Not found in PitchRank: 1 · No current rating: 0 · Data review required: 0</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>MatchBalance seed</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Team name</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Club</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>PowerScore</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>State rank</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>PowerScore seed</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Movement / placement notes</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>Final division</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>Pool</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>Final seed</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>Director notes</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Juniper FC 2016 Blue</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Juniper FC</t>
         </is>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="9" t="n">
         <v>90.10000000000001</v>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>AZ #2</t>
         </is>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F7" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>Seeded</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="inlineStr"/>
-      <c r="I7" s="9" t="inlineStr"/>
-      <c r="J7" s="10" t="inlineStr"/>
-      <c r="K7" s="9" t="inlineStr"/>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Tier 1 · Seeded</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr"/>
+      <c r="I7" s="10" t="inlineStr"/>
+      <c r="J7" s="11" t="inlineStr"/>
+      <c r="K7" s="10" t="inlineStr"/>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="11" t="n">
+      <c r="A8" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Copper State 2016</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>Copper State</t>
         </is>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="14" t="n">
         <v>87.2</v>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>AZ #6</t>
         </is>
       </c>
-      <c r="F8" s="11" t="n">
+      <c r="F8" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="G8" s="12" t="inlineStr">
-        <is>
-          <t>Seeded</t>
-        </is>
-      </c>
-      <c r="H8" s="9" t="inlineStr"/>
-      <c r="I8" s="9" t="inlineStr"/>
-      <c r="J8" s="10" t="inlineStr"/>
-      <c r="K8" s="9" t="inlineStr"/>
-    </row>
-    <row r="9" ht="75" customHeight="1">
-      <c r="A9" s="14" t="n">
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>Tier 1 · Seeded</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr"/>
+      <c r="I8" s="10" t="inlineStr"/>
+      <c r="J8" s="11" t="inlineStr"/>
+      <c r="K8" s="10" t="inlineStr"/>
+    </row>
+    <row r="9" ht="105" customHeight="1">
+      <c r="A9" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>Desert United 2016</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>Desert United</t>
         </is>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D9" s="17" t="n">
         <v>84.59999999999999</v>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>AZ #11</t>
         </is>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="F9" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="G9" s="15" t="inlineStr">
-        <is>
-          <t>Competitive Break: projected matchup quality worsens between seeds 3 and 4; PowerScore difference 11.7 points. · Very close: seeds 1-3 · Seeded</t>
-        </is>
-      </c>
-      <c r="H9" s="17" t="inlineStr"/>
-      <c r="I9" s="17" t="inlineStr"/>
-      <c r="J9" s="18" t="inlineStr"/>
-      <c r="K9" s="17" t="inlineStr"/>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Tier 1 · Competitive Break: projected matchup quality worsens between seeds 3 and 4; PowerScore difference 11.7 points. · Competitive Break: natural strength separation · Very close: seeds 1-3 · Seeded</t>
+        </is>
+      </c>
+      <c r="H9" s="18" t="inlineStr"/>
+      <c r="I9" s="18" t="inlineStr"/>
+      <c r="J9" s="19" t="inlineStr"/>
+      <c r="K9" s="18" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="11" t="n">
+      <c r="A10" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Valley Athletic 2016</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>Valley Athletic</t>
         </is>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="14" t="n">
         <v>72.89999999999999</v>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>AZ #24</t>
         </is>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="G10" s="12" t="inlineStr">
-        <is>
-          <t>Seeded</t>
-        </is>
-      </c>
-      <c r="H10" s="9" t="inlineStr"/>
-      <c r="I10" s="9" t="inlineStr"/>
-      <c r="J10" s="10" t="inlineStr"/>
-      <c r="K10" s="9" t="inlineStr"/>
-    </row>
-    <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="6" t="n">
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>Tier 1 · Seeded</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr"/>
+      <c r="I10" s="10" t="inlineStr"/>
+      <c r="J10" s="11" t="inlineStr"/>
+      <c r="K10" s="10" t="inlineStr"/>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Mesa Juniors 2016</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Mesa Juniors</t>
         </is>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="9" t="n">
         <v>70.09999999999999</v>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>AZ #32</t>
         </is>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>Very close: seeds 4-5 · Seeded</t>
-        </is>
-      </c>
-      <c r="H11" s="9" t="inlineStr"/>
-      <c r="I11" s="9" t="inlineStr"/>
-      <c r="J11" s="10" t="inlineStr"/>
-      <c r="K11" s="9" t="inlineStr"/>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Tier 1 · Very close: seeds 4-5 · Seeded</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr"/>
+      <c r="I11" s="10" t="inlineStr"/>
+      <c r="J11" s="11" t="inlineStr"/>
+      <c r="K11" s="10" t="inlineStr"/>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="11" t="n"/>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Sample Academy 2016</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>Sample Academy</t>
         </is>
       </c>
-      <c r="D12" s="11" t="n"/>
-      <c r="E12" s="11" t="inlineStr"/>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="12" t="inlineStr">
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="12" t="inlineStr"/>
+      <c r="F12" s="12" t="n"/>
+      <c r="G12" s="13" t="inlineStr">
         <is>
           <t>Not found in PitchRank</t>
         </is>
       </c>
-      <c r="H12" s="9" t="inlineStr"/>
-      <c r="I12" s="9" t="inlineStr"/>
-      <c r="J12" s="10" t="inlineStr"/>
-      <c r="K12" s="9" t="inlineStr"/>
+      <c r="H12" s="10" t="inlineStr"/>
+      <c r="I12" s="10" t="inlineStr"/>
+      <c r="J12" s="11" t="inlineStr"/>
+      <c r="K12" s="10" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -886,21 +889,61 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="19" t="inlineStr">
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>Review-required compromise: Tier 1: seeds 1-5 (5 teams; compatible pools 5; minimum 4 games). Pool memberships remain the director's decision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>5 of 6 teams assessed in the tier order; 1 still need placement. These breaks cover the assessed subset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>Review-required compromise: every evaluated arrangement retains projected mismatches.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>Worst remaining mismatch: Juniper FC 2016 Blue vs Mesa Juniors 2016; expected absolute goal difference 4.00, four-goal margin probability 55%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" s="20" t="inlineStr">
+        <is>
+          <t>Formats use the saved MatchBalance profile; confirm game guarantees and event logistics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="20" t="inlineStr">
         <is>
           <t>Sample workbook: use the yellow columns for the director's final decisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="11">
+    <mergeCell ref="A18:K18"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A20:K20"/>
     <mergeCell ref="A15:K15"/>
     <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A16:K16"/>
+    <mergeCell ref="A19:K19"/>
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A17:K17"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D11">
     <cfRule type="dataBar" priority="1">
@@ -933,7 +976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -966,7 +1009,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark boundaries where nearby projected matchups meaningfully worsen; the PowerScore difference is supporting context; they do not assign divisions or pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
+          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark boundaries where nearby projected matchups meaningfully worsen; the PowerScore difference is supporting context; they do not assign divisions or pools. Recommended tier breaks use practical division sizes and all potential matchups. A tier can contain multiple pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
         </is>
       </c>
     </row>
@@ -977,311 +1020,311 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Seeded: 6 · Not found in PitchRank: 0 · No current rating: 0 · Data review required: 1</t>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Suggested tiers: 3 + 3 teams. Seeded: 6 · Not found in PitchRank: 0 · No current rating: 0 · Data review required: 1</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>MatchBalance seed</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Team name</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Club</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>PowerScore</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>State rank</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>PowerScore seed</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>Movement / placement notes</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>Final division</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>Pool</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>Final seed</t>
         </is>
       </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>Director notes</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>Summit SC 2014 Green</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>Summit SC</t>
         </is>
       </c>
-      <c r="D7" s="8" t="n">
+      <c r="D7" s="9" t="n">
         <v>89.3</v>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>CO #4</t>
         </is>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F7" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>Seeded</t>
-        </is>
-      </c>
-      <c r="H7" s="9" t="inlineStr"/>
-      <c r="I7" s="9" t="inlineStr"/>
-      <c r="J7" s="10" t="inlineStr"/>
-      <c r="K7" s="9" t="inlineStr"/>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Tier 1 · Seeded</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr"/>
+      <c r="I7" s="10" t="inlineStr"/>
+      <c r="J7" s="11" t="inlineStr"/>
+      <c r="K7" s="10" t="inlineStr"/>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="11" t="n">
+      <c r="A8" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Front Range FC 2014</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>Front Range FC</t>
         </is>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="14" t="n">
         <v>86.5</v>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>CO #9</t>
         </is>
       </c>
-      <c r="F8" s="11" t="n">
+      <c r="F8" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="G8" s="12" t="inlineStr">
-        <is>
-          <t>Seeded</t>
-        </is>
-      </c>
-      <c r="H8" s="9" t="inlineStr"/>
-      <c r="I8" s="9" t="inlineStr"/>
-      <c r="J8" s="10" t="inlineStr"/>
-      <c r="K8" s="9" t="inlineStr"/>
-    </row>
-    <row r="9" ht="75" customHeight="1">
-      <c r="A9" s="14" t="n">
+      <c r="G8" s="13" t="inlineStr">
+        <is>
+          <t>Tier 1 · Seeded</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr"/>
+      <c r="I8" s="10" t="inlineStr"/>
+      <c r="J8" s="11" t="inlineStr"/>
+      <c r="K8" s="10" t="inlineStr"/>
+    </row>
+    <row r="9" ht="105" customHeight="1">
+      <c r="A9" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>Aspen Athletic 2014</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>Aspen Athletic</t>
         </is>
       </c>
-      <c r="D9" s="16" t="n">
+      <c r="D9" s="17" t="n">
         <v>83.89999999999999</v>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>CO #15</t>
         </is>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="F9" s="15" t="n">
         <v>3</v>
       </c>
-      <c r="G9" s="15" t="inlineStr">
-        <is>
-          <t>Competitive Break: projected matchup quality worsens between seeds 3 and 4; PowerScore difference 12.3 points. · Very close: seeds 1-3 · Seeded</t>
-        </is>
-      </c>
-      <c r="H9" s="17" t="inlineStr"/>
-      <c r="I9" s="17" t="inlineStr"/>
-      <c r="J9" s="18" t="inlineStr"/>
-      <c r="K9" s="17" t="inlineStr"/>
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>Tier 1 · Competitive Break: projected matchup quality worsens between seeds 3 and 4; PowerScore difference 12.3 points. · Recommended tier break + natural strength separation · Very close: seeds 1-3 · Seeded</t>
+        </is>
+      </c>
+      <c r="H9" s="18" t="inlineStr"/>
+      <c r="I9" s="18" t="inlineStr"/>
+      <c r="J9" s="19" t="inlineStr"/>
+      <c r="K9" s="18" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="11" t="n">
+      <c r="A10" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Peak United 2014</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>Peak United</t>
         </is>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="14" t="n">
         <v>71.59999999999999</v>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>CO #29</t>
         </is>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="G10" s="12" t="inlineStr">
-        <is>
-          <t>Seeded</t>
-        </is>
-      </c>
-      <c r="H10" s="9" t="inlineStr"/>
-      <c r="I10" s="9" t="inlineStr"/>
-      <c r="J10" s="10" t="inlineStr"/>
-      <c r="K10" s="9" t="inlineStr"/>
+      <c r="G10" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 · Seeded</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr"/>
+      <c r="I10" s="10" t="inlineStr"/>
+      <c r="J10" s="11" t="inlineStr"/>
+      <c r="K10" s="10" t="inlineStr"/>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="6" t="n">
+      <c r="A11" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>Foothills FC 2014
 Listed: Premier</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>Foothills FC</t>
         </is>
       </c>
-      <c r="D11" s="8" t="n">
+      <c r="D11" s="9" t="n">
         <v>68.89999999999999</v>
       </c>
-      <c r="E11" s="6" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>CO #37</t>
         </is>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>Seeded</t>
-        </is>
-      </c>
-      <c r="H11" s="9" t="inlineStr"/>
-      <c r="I11" s="9" t="inlineStr"/>
-      <c r="J11" s="10" t="inlineStr"/>
-      <c r="K11" s="9" t="inlineStr"/>
-    </row>
-    <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="11" t="n">
+      <c r="G11" s="8" t="inlineStr">
+        <is>
+          <t>Tier 2 · Seeded</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr"/>
+      <c r="I11" s="10" t="inlineStr"/>
+      <c r="J11" s="11" t="inlineStr"/>
+      <c r="K11" s="10" t="inlineStr"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Sample Select 2014</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>Sample Select</t>
         </is>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="14" t="n">
         <v>67.40000000000001</v>
       </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="E12" s="12" t="inlineStr">
         <is>
           <t>CO #42</t>
         </is>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="F12" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="G12" s="12" t="inlineStr">
-        <is>
-          <t>Very close: seeds 4-6 · Seeded</t>
-        </is>
-      </c>
-      <c r="H12" s="9" t="inlineStr"/>
-      <c r="I12" s="9" t="inlineStr"/>
-      <c r="J12" s="10" t="inlineStr"/>
-      <c r="K12" s="9" t="inlineStr"/>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>Tier 2 · Very close: seeds 4-6 · Seeded</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr"/>
+      <c r="I12" s="10" t="inlineStr"/>
+      <c r="J12" s="11" t="inlineStr"/>
+      <c r="K12" s="10" t="inlineStr"/>
     </row>
     <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="6" t="n"/>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="A13" s="7" t="n"/>
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Review United 2014</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>Review United</t>
         </is>
       </c>
-      <c r="D13" s="8" t="n">
+      <c r="D13" s="9" t="n">
         <v>65</v>
       </c>
-      <c r="E13" s="6" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>CO #50</t>
         </is>
       </c>
-      <c r="F13" s="6" t="n"/>
-      <c r="G13" s="7" t="inlineStr">
+      <c r="F13" s="7" t="n"/>
+      <c r="G13" s="8" t="inlineStr">
         <is>
           <t>Data review required</t>
         </is>
       </c>
-      <c r="H13" s="9" t="inlineStr"/>
-      <c r="I13" s="9" t="inlineStr"/>
-      <c r="J13" s="10" t="inlineStr"/>
-      <c r="K13" s="9" t="inlineStr"/>
+      <c r="H13" s="10" t="inlineStr"/>
+      <c r="I13" s="10" t="inlineStr"/>
+      <c r="J13" s="11" t="inlineStr"/>
+      <c r="K13" s="10" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1290,21 +1333,45 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="19" t="inlineStr">
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>Suggested tiers: Tier 1: seeds 1-3 (3 teams; compatible pools 3; minimum 2 games); Tier 2: seeds 4-6 (3 teams; compatible pools 3; minimum 2 games). Pool memberships remain the director's decision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="20" t="inlineStr">
+        <is>
+          <t>6 of 7 teams assessed in the tier order; 1 still need placement. These breaks cover the assessed subset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>Formats use the saved MatchBalance profile; confirm game guarantees and event logistics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>Sample data only. Strength markers are observations, not automatic divisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="9">
+    <mergeCell ref="A18:K18"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A16:K16"/>
+    <mergeCell ref="A19:K19"/>
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A17:K17"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D12">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
Expand MatchBalance formats with automatic cohort guidance
</commit_message>
<xml_diff>
--- a/docs/design/matchbalance-excel/director-workbook-sample.xlsx
+++ b/docs/design/matchbalance-excel/director-workbook-sample.xlsx
@@ -14,7 +14,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'U10 Boys'!$1:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$K$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'U12 Girls'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$K$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$K$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -892,7 +892,7 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="20" t="inlineStr">
         <is>
-          <t>Review-required compromise: Tier 1: seeds 1-5 (5 teams; compatible pools 5; minimum 4 games). Pool memberships remain the director's decision.</t>
+          <t>Tier 1: seeds 1-5 (5 teams; Partial round robin; 3 guaranteed; up to 4 games; 8 matches total; no playoffs; Use points per game for unequal preliminary game counts; all played games still count toward the game guarantee.; compatible pools 5)</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1336,36 +1336,44 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>Suggested tiers: Tier 1: seeds 1-3 (3 teams; compatible pools 3; minimum 2 games); Tier 2: seeds 4-6 (3 teams; compatible pools 3; minimum 2 games). Pool memberships remain the director's decision.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1">
+          <t>Tier 1: seeds 1-3 (3 teams; Round robin, extra points match and final; 3 guaranteed; up to 4 games; 5 matches total; opponents may meet up to 2 times; includes playoffs; compatible pools 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
       <c r="A17" s="20" t="inlineStr">
         <is>
-          <t>6 of 7 teams assessed in the tier order; 1 still need placement. These breaks cover the assessed subset.</t>
+          <t>Tier 2: seeds 4-6 (3 teams; Round robin, extra points match and final; 3 guaranteed; up to 4 games; 5 matches total; opponents may meet up to 2 times; includes playoffs; compatible pools 3)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>Formats use the saved MatchBalance profile; confirm game guarantees and event logistics.</t>
+          <t>6 of 7 teams assessed in the tier order; 1 still need placement. These breaks cover the assessed subset.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="20" t="inlineStr">
         <is>
+          <t>Formats use the saved MatchBalance profile; confirm game guarantees and event logistics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
           <t>Sample data only. Strength markers are observations, not automatic divisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A18:K18"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A20:K20"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A16:K16"/>
     <mergeCell ref="A19:K19"/>

</xml_diff>

<commit_message>
Expand MatchBalance formats with automatic cohort guidance (#1263)
</commit_message>
<xml_diff>
--- a/docs/design/matchbalance-excel/director-workbook-sample.xlsx
+++ b/docs/design/matchbalance-excel/director-workbook-sample.xlsx
@@ -14,7 +14,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'U10 Boys'!$1:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$K$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'U12 Girls'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$K$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$K$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -892,7 +892,7 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="20" t="inlineStr">
         <is>
-          <t>Review-required compromise: Tier 1: seeds 1-5 (5 teams; compatible pools 5; minimum 4 games). Pool memberships remain the director's decision.</t>
+          <t>Tier 1: seeds 1-5 (5 teams; Partial round robin; 3 guaranteed; up to 4 games; 8 matches total; no playoffs; Use points per game for unequal preliminary game counts; all played games still count toward the game guarantee.; compatible pools 5)</t>
         </is>
       </c>
     </row>
@@ -976,7 +976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1336,36 +1336,44 @@
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>Suggested tiers: Tier 1: seeds 1-3 (3 teams; compatible pools 3; minimum 2 games); Tier 2: seeds 4-6 (3 teams; compatible pools 3; minimum 2 games). Pool memberships remain the director's decision.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1">
+          <t>Tier 1: seeds 1-3 (3 teams; Round robin, extra points match and final; 3 guaranteed; up to 4 games; 5 matches total; opponents may meet up to 2 times; includes playoffs; compatible pools 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
       <c r="A17" s="20" t="inlineStr">
         <is>
-          <t>6 of 7 teams assessed in the tier order; 1 still need placement. These breaks cover the assessed subset.</t>
+          <t>Tier 2: seeds 4-6 (3 teams; Round robin, extra points match and final; 3 guaranteed; up to 4 games; 5 matches total; opponents may meet up to 2 times; includes playoffs; compatible pools 3)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>Formats use the saved MatchBalance profile; confirm game guarantees and event logistics.</t>
+          <t>6 of 7 teams assessed in the tier order; 1 still need placement. These breaks cover the assessed subset.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="20" t="inlineStr">
         <is>
+          <t>Formats use the saved MatchBalance profile; confirm game guarantees and event logistics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
           <t>Sample data only. Strength markers are observations, not automatic divisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A18:K18"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A3:K3"/>
+    <mergeCell ref="A20:K20"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A16:K16"/>
     <mergeCell ref="A19:K19"/>

</xml_diff>

<commit_message>
Prefer practical strength divisions and track ordering implementation changes
</commit_message>
<xml_diff>
--- a/docs/design/matchbalance-excel/director-workbook-sample.xlsx
+++ b/docs/design/matchbalance-excel/director-workbook-sample.xlsx
@@ -14,7 +14,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'U10 Boys'!$1:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$K$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'U12 Girls'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$K$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$K$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -976,7 +976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1354,26 +1354,34 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1">
+    <row r="19" ht="30" customHeight="1">
       <c r="A19" s="20" t="inlineStr">
         <is>
-          <t>Formats use the saved MatchBalance profile; confirm game guarantees and event logistics.</t>
+          <t>Small-division fallback: no complete, fully assessed arrangement with every strength division at least 4 teams passes the competitive limits and format restrictions. Smaller pools inside a larger strength division are still allowed.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="20" t="inlineStr">
         <is>
+          <t>Formats use the saved MatchBalance profile; confirm game guarantees and event logistics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
           <t>Sample data only. Strength markers are observations, not automatic divisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A18:K18"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A20:K20"/>
+    <mergeCell ref="A21:K21"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A16:K16"/>
     <mergeCell ref="A19:K19"/>

</xml_diff>

<commit_message>
Add MatchBalance ordering previews and practical tier guidance (#1323)
* Add evidence-based MatchBalance ordering previews and safe cohort intake

* Prefer practical strength divisions and track ordering implementation changes
</commit_message>
<xml_diff>
--- a/docs/design/matchbalance-excel/director-workbook-sample.xlsx
+++ b/docs/design/matchbalance-excel/director-workbook-sample.xlsx
@@ -14,7 +14,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'U10 Boys'!$1:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$K$20</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'U12 Girls'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$K$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$K$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -976,7 +976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1354,26 +1354,34 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1">
+    <row r="19" ht="30" customHeight="1">
       <c r="A19" s="20" t="inlineStr">
         <is>
-          <t>Formats use the saved MatchBalance profile; confirm game guarantees and event logistics.</t>
+          <t>Small-division fallback: no complete, fully assessed arrangement with every strength division at least 4 teams passes the competitive limits and format restrictions. Smaller pools inside a larger strength division are still allowed.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="20" t="inlineStr">
         <is>
+          <t>Formats use the saved MatchBalance profile; confirm game guarantees and event logistics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="20" t="inlineStr">
+        <is>
           <t>Sample data only. Strength markers are observations, not automatic divisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A18:K18"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A3:K3"/>
     <mergeCell ref="A20:K20"/>
+    <mergeCell ref="A21:K21"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A16:K16"/>
     <mergeCell ref="A19:K19"/>

</xml_diff>

<commit_message>
Use game evidence for MatchBalance seed order and practical tier guidance
</commit_message>
<xml_diff>
--- a/docs/design/matchbalance-excel/director-workbook-sample.xlsx
+++ b/docs/design/matchbalance-excel/director-workbook-sample.xlsx
@@ -607,7 +607,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark boundaries where nearby projected matchups meaningfully worsen; the PowerScore difference is supporting context; they do not assign divisions or pools. Recommended tier breaks use practical division sizes and all potential matchups. A tier can contain multiple pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
+          <t>Read from seed 1 down. Tier lines suggest strength divisions; a division can contain several pools. Natural separation marks a strength gap; practical splits also consider usable division sizes. Review warnings and unplaced teams before making final placements.</t>
         </is>
       </c>
     </row>
@@ -857,7 +857,7 @@
       <c r="J11" s="11" t="inlineStr"/>
       <c r="K11" s="10" t="inlineStr"/>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="30" customHeight="1">
       <c r="A12" s="12" t="n"/>
       <c r="B12" s="13" t="inlineStr">
         <is>
@@ -874,7 +874,7 @@
       <c r="F12" s="12" t="n"/>
       <c r="G12" s="13" t="inlineStr">
         <is>
-          <t>Not found in PitchRank</t>
+          <t>Not found in PitchRank. · Not found in PitchRank</t>
         </is>
       </c>
       <c r="H12" s="10" t="inlineStr"/>
@@ -906,7 +906,7 @@
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="20" t="inlineStr">
         <is>
-          <t>Review-required compromise: every evaluated arrangement retains projected mismatches.</t>
+          <t>Review-required compromise: this split retains projected mismatches.</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark boundaries where nearby projected matchups meaningfully worsen; the PowerScore difference is supporting context; they do not assign divisions or pools. Recommended tier breaks use practical division sizes and all potential matchups. A tier can contain multiple pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
+          <t>Read from seed 1 down. Tier lines suggest strength divisions; a division can contain several pools. Natural separation marks a strength gap; practical splits also consider usable division sizes. Review warnings and unplaced teams before making final placements.</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       <c r="J12" s="11" t="inlineStr"/>
       <c r="K12" s="10" t="inlineStr"/>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13" ht="45" customHeight="1">
       <c r="A13" s="7" t="n"/>
       <c r="B13" s="8" t="inlineStr">
         <is>
@@ -1318,7 +1318,7 @@
       <c r="F13" s="7" t="n"/>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>Data review required</t>
+          <t>Confirm the team identity before seeding. · Data review required</t>
         </is>
       </c>
       <c r="H13" s="10" t="inlineStr"/>

</xml_diff>

<commit_message>
Simplify MatchBalance director sheets while preserving review warnings
</commit_message>
<xml_diff>
--- a/docs/design/matchbalance-excel/director-workbook-sample.xlsx
+++ b/docs/design/matchbalance-excel/director-workbook-sample.xlsx
@@ -12,9 +12,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'U10 Boys'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$K$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$K$18</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'U12 Girls'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$K$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$K$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -255,7 +255,7 @@
     <tableColumn id="4" name="PowerScore"/>
     <tableColumn id="5" name="State rank"/>
     <tableColumn id="6" name="PowerScore seed"/>
-    <tableColumn id="7" name="Movement / placement notes"/>
+    <tableColumn id="7" name="Tier / placement"/>
     <tableColumn id="8" name="Final division"/>
     <tableColumn id="9" name="Pool"/>
     <tableColumn id="10" name="Final seed"/>
@@ -275,7 +275,7 @@
     <tableColumn id="4" name="PowerScore"/>
     <tableColumn id="5" name="State rank"/>
     <tableColumn id="6" name="PowerScore seed"/>
-    <tableColumn id="7" name="Movement / placement notes"/>
+    <tableColumn id="7" name="Tier / placement"/>
     <tableColumn id="8" name="Final division"/>
     <tableColumn id="9" name="Pool"/>
     <tableColumn id="10" name="Final seed"/>
@@ -574,7 +574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -658,7 +658,7 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Movement / placement notes</t>
+          <t>Tier / placement</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -709,7 +709,7 @@
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>Tier 1 · Seeded</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="H7" s="10" t="inlineStr"/>
@@ -744,7 +744,7 @@
       </c>
       <c r="G8" s="13" t="inlineStr">
         <is>
-          <t>Tier 1 · Seeded</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="H8" s="10" t="inlineStr"/>
@@ -752,7 +752,7 @@
       <c r="J8" s="11" t="inlineStr"/>
       <c r="K8" s="10" t="inlineStr"/>
     </row>
-    <row r="9" ht="105" customHeight="1">
+    <row r="9" ht="15" customHeight="1">
       <c r="A9" s="15" t="n">
         <v>3</v>
       </c>
@@ -779,7 +779,7 @@
       </c>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>Tier 1 · Competitive Break: projected matchup quality worsens between seeds 3 and 4; PowerScore difference 11.7 points. · Competitive Break: natural strength separation · Very close: seeds 1-3 · Seeded</t>
+          <t>Tier 1 · Strength gap below</t>
         </is>
       </c>
       <c r="H9" s="18" t="inlineStr"/>
@@ -814,7 +814,7 @@
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>Tier 1 · Seeded</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="H10" s="10" t="inlineStr"/>
@@ -822,7 +822,7 @@
       <c r="J10" s="11" t="inlineStr"/>
       <c r="K10" s="10" t="inlineStr"/>
     </row>
-    <row r="11" ht="30" customHeight="1">
+    <row r="11" ht="15" customHeight="1">
       <c r="A11" s="7" t="n">
         <v>5</v>
       </c>
@@ -849,7 +849,7 @@
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>Tier 1 · Very close: seeds 4-5 · Seeded</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="H11" s="10" t="inlineStr"/>
@@ -874,7 +874,7 @@
       <c r="F12" s="12" t="n"/>
       <c r="G12" s="13" t="inlineStr">
         <is>
-          <t>Not found in PitchRank. · Not found in PitchRank</t>
+          <t>Not found in PitchRank · Not found in PitchRank.</t>
         </is>
       </c>
       <c r="H12" s="10" t="inlineStr"/>
@@ -892,55 +892,39 @@
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="20" t="inlineStr">
         <is>
-          <t>Tier 1: seeds 1-5 (5 teams; Partial round robin; 3 guaranteed; up to 4 games; 8 matches total; no playoffs; Use points per game for unequal preliminary game counts; all played games still count toward the game guarantee.; compatible pools 5)</t>
+          <t>Tier 1 — 5 teams: Partial round robin; 3 guaranteed, up to 4 games; 8 matches; unequal preliminary games — confirm scheduling and standings rules</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>5 of 6 teams assessed in the tier order; 1 still need placement. These breaks cover the assessed subset.</t>
+          <t>Matchup review needed: this split still includes potentially uneven games.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="20" t="inlineStr">
         <is>
-          <t>Review-required compromise: this split retains projected mismatches.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
+          <t>Review this matchup: Juniper FC 2016 Blue vs Mesa Juniors 2016; projected goal gap 4.00, chance of a 4+ goal margin 55%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>Worst remaining mismatch: Juniper FC 2016 Blue vs Mesa Juniors 2016; expected absolute goal difference 4.00, four-goal margin probability 55%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="20" t="inlineStr">
-        <is>
-          <t>Formats use the saved MatchBalance profile; confirm game guarantees and event logistics.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="20" t="inlineStr">
-        <is>
           <t>Sample workbook: use the yellow columns for the director's final decisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="9">
     <mergeCell ref="A18:K18"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A20:K20"/>
     <mergeCell ref="A15:K15"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A16:K16"/>
-    <mergeCell ref="A19:K19"/>
     <mergeCell ref="A5:K5"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A17:K17"/>
@@ -976,7 +960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1060,7 +1044,7 @@
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Movement / placement notes</t>
+          <t>Tier / placement</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -1111,7 +1095,7 @@
       </c>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>Tier 1 · Seeded</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="H7" s="10" t="inlineStr"/>
@@ -1146,7 +1130,7 @@
       </c>
       <c r="G8" s="13" t="inlineStr">
         <is>
-          <t>Tier 1 · Seeded</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="H8" s="10" t="inlineStr"/>
@@ -1154,7 +1138,7 @@
       <c r="J8" s="11" t="inlineStr"/>
       <c r="K8" s="10" t="inlineStr"/>
     </row>
-    <row r="9" ht="105" customHeight="1">
+    <row r="9" ht="15" customHeight="1">
       <c r="A9" s="15" t="n">
         <v>3</v>
       </c>
@@ -1181,7 +1165,7 @@
       </c>
       <c r="G9" s="16" t="inlineStr">
         <is>
-          <t>Tier 1 · Competitive Break: projected matchup quality worsens between seeds 3 and 4; PowerScore difference 12.3 points. · Recommended tier break + natural strength separation · Very close: seeds 1-3 · Seeded</t>
+          <t>Tier 1 · Strength gap below</t>
         </is>
       </c>
       <c r="H9" s="18" t="inlineStr"/>
@@ -1216,7 +1200,7 @@
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>Tier 2 · Seeded</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="H10" s="10" t="inlineStr"/>
@@ -1252,7 +1236,7 @@
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>Tier 2 · Seeded</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="H11" s="10" t="inlineStr"/>
@@ -1260,7 +1244,7 @@
       <c r="J11" s="11" t="inlineStr"/>
       <c r="K11" s="10" t="inlineStr"/>
     </row>
-    <row r="12" ht="30" customHeight="1">
+    <row r="12" ht="15" customHeight="1">
       <c r="A12" s="12" t="n">
         <v>6</v>
       </c>
@@ -1287,7 +1271,7 @@
       </c>
       <c r="G12" s="13" t="inlineStr">
         <is>
-          <t>Tier 2 · Very close: seeds 4-6 · Seeded</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="H12" s="10" t="inlineStr"/>
@@ -1318,7 +1302,7 @@
       <c r="F13" s="7" t="n"/>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>Confirm the team identity before seeding. · Data review required</t>
+          <t>Data review required · Confirm the team identity before seeding.</t>
         </is>
       </c>
       <c r="H13" s="10" t="inlineStr"/>
@@ -1333,55 +1317,39 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1">
+    <row r="16" ht="15" customHeight="1">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>Tier 1: seeds 1-3 (3 teams; Round robin, extra points match and final; 3 guaranteed; up to 4 games; 5 matches total; opponents may meet up to 2 times; includes playoffs; compatible pools 3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
+          <t>Tier 1 — 3 teams: Round robin, extra points match and final; 3 guaranteed, up to 4 games; 5 matches; repeat opponents possible</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
       <c r="A17" s="20" t="inlineStr">
         <is>
-          <t>Tier 2: seeds 4-6 (3 teams; Round robin, extra points match and final; 3 guaranteed; up to 4 games; 5 matches total; opponents may meet up to 2 times; includes playoffs; compatible pools 3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1">
+          <t>Tier 2 — 3 teams: Round robin, extra points match and final; 3 guaranteed, up to 4 games; 5 matches; repeat opponents possible</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>6 of 7 teams assessed in the tier order; 1 still need placement. These breaks cover the assessed subset.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
+          <t>Small-division fallback: no complete, fully assessed arrangement with every strength division at least 4 teams passes the competitive limits and format restrictions. Smaller pools inside a larger strength division are still allowed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="15" customHeight="1">
       <c r="A19" s="20" t="inlineStr">
         <is>
-          <t>Small-division fallback: no complete, fully assessed arrangement with every strength division at least 4 teams passes the competitive limits and format restrictions. Smaller pools inside a larger strength division are still allowed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="20" t="inlineStr">
-        <is>
-          <t>Formats use the saved MatchBalance profile; confirm game guarantees and event logistics.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="20" t="inlineStr">
-        <is>
           <t>Sample data only. Strength markers are observations, not automatic divisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="9">
     <mergeCell ref="A18:K18"/>
     <mergeCell ref="A4:K4"/>
     <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A20:K20"/>
-    <mergeCell ref="A21:K21"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A16:K16"/>
     <mergeCell ref="A19:K19"/>

</xml_diff>

<commit_message>
Restore MatchBalance sheet details and yellow competitive breaks
</commit_message>
<xml_diff>
--- a/docs/design/matchbalance-excel/director-workbook-sample.xlsx
+++ b/docs/design/matchbalance-excel/director-workbook-sample.xlsx
@@ -12,9 +12,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'U10 Boys'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$K$18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$L$18</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'U12 Girls'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$K$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$L$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -246,9 +246,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Cohort1" displayName="Cohort1" ref="A6:K12" headerRowCount="1">
-  <autoFilter ref="A6:K12"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Cohort1" displayName="Cohort1" ref="A6:L12" headerRowCount="1">
+  <autoFilter ref="A6:L12"/>
+  <tableColumns count="12">
     <tableColumn id="1" name="MatchBalance seed"/>
     <tableColumn id="2" name="Team name"/>
     <tableColumn id="3" name="Club"/>
@@ -260,15 +260,16 @@
     <tableColumn id="9" name="Pool"/>
     <tableColumn id="10" name="Final seed"/>
     <tableColumn id="11" name="Director notes"/>
+    <tableColumn id="12" name="Record (W-L-D)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Cohort2" displayName="Cohort2" ref="A6:K13" headerRowCount="1">
-  <autoFilter ref="A6:K13"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Cohort2" displayName="Cohort2" ref="A6:L13" headerRowCount="1">
+  <autoFilter ref="A6:L13"/>
+  <tableColumns count="12">
     <tableColumn id="1" name="MatchBalance seed"/>
     <tableColumn id="2" name="Team name"/>
     <tableColumn id="3" name="Club"/>
@@ -280,6 +281,7 @@
     <tableColumn id="9" name="Pool"/>
     <tableColumn id="10" name="Final seed"/>
     <tableColumn id="11" name="Director notes"/>
+    <tableColumn id="12" name="Record (W-L-D)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -574,7 +576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -588,6 +590,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -681,6 +684,11 @@
           <t>Director notes</t>
         </is>
       </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>Record (W-L-D)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="7" t="n">
@@ -716,6 +724,7 @@
       <c r="I7" s="10" t="inlineStr"/>
       <c r="J7" s="11" t="inlineStr"/>
       <c r="K7" s="10" t="inlineStr"/>
+      <c r="L7" s="7" t="inlineStr"/>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="12" t="n">
@@ -751,6 +760,7 @@
       <c r="I8" s="10" t="inlineStr"/>
       <c r="J8" s="11" t="inlineStr"/>
       <c r="K8" s="10" t="inlineStr"/>
+      <c r="L8" s="7" t="inlineStr"/>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="15" t="n">
@@ -786,6 +796,7 @@
       <c r="I9" s="18" t="inlineStr"/>
       <c r="J9" s="19" t="inlineStr"/>
       <c r="K9" s="18" t="inlineStr"/>
+      <c r="L9" s="15" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="12" t="n">
@@ -821,6 +832,7 @@
       <c r="I10" s="10" t="inlineStr"/>
       <c r="J10" s="11" t="inlineStr"/>
       <c r="K10" s="10" t="inlineStr"/>
+      <c r="L10" s="7" t="inlineStr"/>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="7" t="n">
@@ -856,6 +868,7 @@
       <c r="I11" s="10" t="inlineStr"/>
       <c r="J11" s="11" t="inlineStr"/>
       <c r="K11" s="10" t="inlineStr"/>
+      <c r="L11" s="7" t="inlineStr"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="12" t="n"/>
@@ -881,6 +894,7 @@
       <c r="I12" s="10" t="inlineStr"/>
       <c r="J12" s="11" t="inlineStr"/>
       <c r="K12" s="10" t="inlineStr"/>
+      <c r="L12" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -919,15 +933,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A18:K18"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A15:K15"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A16:K16"/>
-    <mergeCell ref="A5:K5"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A17:K17"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A16:L16"/>
+    <mergeCell ref="A15:L15"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A17:L17"/>
+    <mergeCell ref="A18:L18"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A4:L4"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D11">
     <cfRule type="dataBar" priority="1">
@@ -960,7 +974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -974,6 +988,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1067,6 +1082,11 @@
           <t>Director notes</t>
         </is>
       </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>Record (W-L-D)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="7" t="n">
@@ -1102,6 +1122,7 @@
       <c r="I7" s="10" t="inlineStr"/>
       <c r="J7" s="11" t="inlineStr"/>
       <c r="K7" s="10" t="inlineStr"/>
+      <c r="L7" s="7" t="inlineStr"/>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="12" t="n">
@@ -1137,6 +1158,7 @@
       <c r="I8" s="10" t="inlineStr"/>
       <c r="J8" s="11" t="inlineStr"/>
       <c r="K8" s="10" t="inlineStr"/>
+      <c r="L8" s="7" t="inlineStr"/>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="15" t="n">
@@ -1172,6 +1194,7 @@
       <c r="I9" s="18" t="inlineStr"/>
       <c r="J9" s="19" t="inlineStr"/>
       <c r="K9" s="18" t="inlineStr"/>
+      <c r="L9" s="15" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="12" t="n">
@@ -1207,6 +1230,7 @@
       <c r="I10" s="10" t="inlineStr"/>
       <c r="J10" s="11" t="inlineStr"/>
       <c r="K10" s="10" t="inlineStr"/>
+      <c r="L10" s="7" t="inlineStr"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="7" t="n">
@@ -1243,6 +1267,7 @@
       <c r="I11" s="10" t="inlineStr"/>
       <c r="J11" s="11" t="inlineStr"/>
       <c r="K11" s="10" t="inlineStr"/>
+      <c r="L11" s="7" t="inlineStr"/>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="12" t="n">
@@ -1278,6 +1303,7 @@
       <c r="I12" s="10" t="inlineStr"/>
       <c r="J12" s="11" t="inlineStr"/>
       <c r="K12" s="10" t="inlineStr"/>
+      <c r="L12" s="7" t="inlineStr"/>
     </row>
     <row r="13" ht="45" customHeight="1">
       <c r="A13" s="7" t="n"/>
@@ -1309,6 +1335,7 @@
       <c r="I13" s="10" t="inlineStr"/>
       <c r="J13" s="11" t="inlineStr"/>
       <c r="K13" s="10" t="inlineStr"/>
+      <c r="L13" s="7" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1347,15 +1374,15 @@
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A18:K18"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A16:K16"/>
-    <mergeCell ref="A19:K19"/>
-    <mergeCell ref="A5:K5"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A17:K17"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A16:L16"/>
+    <mergeCell ref="A19:L19"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A17:L17"/>
+    <mergeCell ref="A18:L18"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A4:L4"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D12">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
Choose practical MatchBalance tiers without overriding safe game evidence
</commit_message>
<xml_diff>
--- a/docs/design/matchbalance-excel/director-workbook-sample.xlsx
+++ b/docs/design/matchbalance-excel/director-workbook-sample.xlsx
@@ -903,10 +903,10 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1">
+    <row r="15" ht="15" customHeight="1">
       <c r="A15" s="20" t="inlineStr">
         <is>
-          <t>Tier 1 — 5 teams: Partial round robin; 3 guaranteed, up to 4 games; 8 matches; unequal preliminary games — confirm scheduling and standings rules</t>
+          <t>Tier 1 — 5 teams: Round robin; 4 games each; 10 matches</t>
         </is>
       </c>
     </row>
@@ -1347,21 +1347,21 @@
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="20" t="inlineStr">
         <is>
-          <t>Tier 1 — 3 teams: Round robin, extra points match and final; 3 guaranteed, up to 4 games; 5 matches; repeat opponents possible</t>
+          <t>Tier 1 — 3 teams: Double round robin; 4 games each; 6 matches; repeat opponents possible</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="20" t="inlineStr">
         <is>
-          <t>Tier 2 — 3 teams: Round robin, extra points match and final; 3 guaranteed, up to 4 games; 5 matches; repeat opponents possible</t>
+          <t>Tier 2 — 3 teams: Double round robin; 4 games each; 6 matches; repeat opponents possible</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>Small-division fallback: no complete, fully assessed arrangement with every strength division at least 4 teams passes the competitive limits and format restrictions. Smaller pools inside a larger strength division are still allowed.</t>
+          <t>Small tier: no equally practical, fully assessed split keeps every tier at least 4 teams, preserves the supported strength breaks, and passes the competitive limits.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Show national cohort ranks instead of seed changes on director sheets
</commit_message>
<xml_diff>
--- a/docs/design/matchbalance-excel/director-workbook-sample.xlsx
+++ b/docs/design/matchbalance-excel/director-workbook-sample.xlsx
@@ -111,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -136,6 +136,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -151,6 +154,9 @@
     <xf numFmtId="164" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -159,6 +165,9 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -254,7 +263,7 @@
     <tableColumn id="3" name="Club"/>
     <tableColumn id="4" name="PowerScore"/>
     <tableColumn id="5" name="State rank"/>
-    <tableColumn id="6" name="PowerScore seed"/>
+    <tableColumn id="6" name="National rank"/>
     <tableColumn id="7" name="Tier / placement"/>
     <tableColumn id="8" name="Final division"/>
     <tableColumn id="9" name="Pool"/>
@@ -275,7 +284,7 @@
     <tableColumn id="3" name="Club"/>
     <tableColumn id="4" name="PowerScore"/>
     <tableColumn id="5" name="State rank"/>
-    <tableColumn id="6" name="PowerScore seed"/>
+    <tableColumn id="6" name="National rank"/>
     <tableColumn id="7" name="Tier / placement"/>
     <tableColumn id="8" name="Final division"/>
     <tableColumn id="9" name="Pool"/>
@@ -656,7 +665,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>PowerScore seed</t>
+          <t>National rank</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -712,126 +721,118 @@
           <t>AZ #2</t>
         </is>
       </c>
-      <c r="F7" s="7" t="n">
-        <v>1</v>
-      </c>
+      <c r="F7" s="10" t="inlineStr"/>
       <c r="G7" s="8" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr"/>
-      <c r="I7" s="10" t="inlineStr"/>
-      <c r="J7" s="11" t="inlineStr"/>
-      <c r="K7" s="10" t="inlineStr"/>
+      <c r="H7" s="11" t="inlineStr"/>
+      <c r="I7" s="11" t="inlineStr"/>
+      <c r="J7" s="12" t="inlineStr"/>
+      <c r="K7" s="11" t="inlineStr"/>
       <c r="L7" s="7" t="inlineStr"/>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>Copper State 2016</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>Copper State</t>
         </is>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="15" t="n">
         <v>87.2</v>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>AZ #6</t>
         </is>
       </c>
-      <c r="F8" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="G8" s="13" t="inlineStr">
+      <c r="F8" s="16" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr"/>
-      <c r="I8" s="10" t="inlineStr"/>
-      <c r="J8" s="11" t="inlineStr"/>
-      <c r="K8" s="10" t="inlineStr"/>
+      <c r="H8" s="11" t="inlineStr"/>
+      <c r="I8" s="11" t="inlineStr"/>
+      <c r="J8" s="12" t="inlineStr"/>
+      <c r="K8" s="11" t="inlineStr"/>
       <c r="L8" s="7" t="inlineStr"/>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="15" t="n">
+      <c r="A9" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>Desert United 2016</t>
         </is>
       </c>
-      <c r="C9" s="16" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>Desert United</t>
         </is>
       </c>
-      <c r="D9" s="17" t="n">
+      <c r="D9" s="19" t="n">
         <v>84.59999999999999</v>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>AZ #11</t>
         </is>
       </c>
-      <c r="F9" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="G9" s="16" t="inlineStr">
+      <c r="F9" s="20" t="inlineStr"/>
+      <c r="G9" s="18" t="inlineStr">
         <is>
           <t>Tier 1 · Strength gap below</t>
         </is>
       </c>
-      <c r="H9" s="18" t="inlineStr"/>
-      <c r="I9" s="18" t="inlineStr"/>
-      <c r="J9" s="19" t="inlineStr"/>
-      <c r="K9" s="18" t="inlineStr"/>
-      <c r="L9" s="15" t="inlineStr"/>
+      <c r="H9" s="21" t="inlineStr"/>
+      <c r="I9" s="21" t="inlineStr"/>
+      <c r="J9" s="22" t="inlineStr"/>
+      <c r="K9" s="21" t="inlineStr"/>
+      <c r="L9" s="17" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="12" t="n">
+      <c r="A10" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>Valley Athletic 2016</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>Valley Athletic</t>
         </is>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="15" t="n">
         <v>72.89999999999999</v>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>AZ #24</t>
         </is>
       </c>
-      <c r="F10" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="G10" s="13" t="inlineStr">
+      <c r="F10" s="16" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="H10" s="10" t="inlineStr"/>
-      <c r="I10" s="10" t="inlineStr"/>
-      <c r="J10" s="11" t="inlineStr"/>
-      <c r="K10" s="10" t="inlineStr"/>
+      <c r="H10" s="11" t="inlineStr"/>
+      <c r="I10" s="11" t="inlineStr"/>
+      <c r="J10" s="12" t="inlineStr"/>
+      <c r="K10" s="11" t="inlineStr"/>
       <c r="L10" s="7" t="inlineStr"/>
     </row>
     <row r="11" ht="15" customHeight="1">
@@ -856,44 +857,42 @@
           <t>AZ #32</t>
         </is>
       </c>
-      <c r="F11" s="7" t="n">
-        <v>5</v>
-      </c>
+      <c r="F11" s="10" t="inlineStr"/>
       <c r="G11" s="8" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="H11" s="10" t="inlineStr"/>
-      <c r="I11" s="10" t="inlineStr"/>
-      <c r="J11" s="11" t="inlineStr"/>
-      <c r="K11" s="10" t="inlineStr"/>
+      <c r="H11" s="11" t="inlineStr"/>
+      <c r="I11" s="11" t="inlineStr"/>
+      <c r="J11" s="12" t="inlineStr"/>
+      <c r="K11" s="11" t="inlineStr"/>
       <c r="L11" s="7" t="inlineStr"/>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="12" t="n"/>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="A12" s="13" t="n"/>
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>Sample Academy 2016</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>Sample Academy</t>
         </is>
       </c>
-      <c r="D12" s="12" t="n"/>
-      <c r="E12" s="12" t="inlineStr"/>
-      <c r="F12" s="12" t="n"/>
-      <c r="G12" s="13" t="inlineStr">
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="13" t="inlineStr"/>
+      <c r="F12" s="16" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
         <is>
           <t>Not found in PitchRank · Not found in PitchRank.</t>
         </is>
       </c>
-      <c r="H12" s="10" t="inlineStr"/>
-      <c r="I12" s="10" t="inlineStr"/>
-      <c r="J12" s="11" t="inlineStr"/>
-      <c r="K12" s="10" t="inlineStr"/>
+      <c r="H12" s="11" t="inlineStr"/>
+      <c r="I12" s="11" t="inlineStr"/>
+      <c r="J12" s="12" t="inlineStr"/>
+      <c r="K12" s="11" t="inlineStr"/>
       <c r="L12" s="7" t="inlineStr"/>
     </row>
     <row r="14">
@@ -904,28 +903,28 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="20" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>Tier 1 — 5 teams: Round robin; 4 games each; 10 matches</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t>Matchup review needed: this split still includes potentially uneven games.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t>Review this matchup: Juniper FC 2016 Blue vs Mesa Juniors 2016; projected goal gap 4.00, chance of a 4+ goal margin 55%.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="20" t="inlineStr">
+      <c r="A18" s="23" t="inlineStr">
         <is>
           <t>Sample workbook: use the yellow columns for the director's final decisions.</t>
         </is>
@@ -1054,7 +1053,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>PowerScore seed</t>
+          <t>National rank</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -1110,126 +1109,118 @@
           <t>CO #4</t>
         </is>
       </c>
-      <c r="F7" s="7" t="n">
-        <v>1</v>
-      </c>
+      <c r="F7" s="10" t="inlineStr"/>
       <c r="G7" s="8" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="H7" s="10" t="inlineStr"/>
-      <c r="I7" s="10" t="inlineStr"/>
-      <c r="J7" s="11" t="inlineStr"/>
-      <c r="K7" s="10" t="inlineStr"/>
+      <c r="H7" s="11" t="inlineStr"/>
+      <c r="I7" s="11" t="inlineStr"/>
+      <c r="J7" s="12" t="inlineStr"/>
+      <c r="K7" s="11" t="inlineStr"/>
       <c r="L7" s="7" t="inlineStr"/>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>Front Range FC 2014</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>Front Range FC</t>
         </is>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="15" t="n">
         <v>86.5</v>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>CO #9</t>
         </is>
       </c>
-      <c r="F8" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="G8" s="13" t="inlineStr">
+      <c r="F8" s="16" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="H8" s="10" t="inlineStr"/>
-      <c r="I8" s="10" t="inlineStr"/>
-      <c r="J8" s="11" t="inlineStr"/>
-      <c r="K8" s="10" t="inlineStr"/>
+      <c r="H8" s="11" t="inlineStr"/>
+      <c r="I8" s="11" t="inlineStr"/>
+      <c r="J8" s="12" t="inlineStr"/>
+      <c r="K8" s="11" t="inlineStr"/>
       <c r="L8" s="7" t="inlineStr"/>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="15" t="n">
+      <c r="A9" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>Aspen Athletic 2014</t>
         </is>
       </c>
-      <c r="C9" s="16" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>Aspen Athletic</t>
         </is>
       </c>
-      <c r="D9" s="17" t="n">
+      <c r="D9" s="19" t="n">
         <v>83.89999999999999</v>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>CO #15</t>
         </is>
       </c>
-      <c r="F9" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="G9" s="16" t="inlineStr">
+      <c r="F9" s="20" t="inlineStr"/>
+      <c r="G9" s="18" t="inlineStr">
         <is>
           <t>Tier 1 · Strength gap below</t>
         </is>
       </c>
-      <c r="H9" s="18" t="inlineStr"/>
-      <c r="I9" s="18" t="inlineStr"/>
-      <c r="J9" s="19" t="inlineStr"/>
-      <c r="K9" s="18" t="inlineStr"/>
-      <c r="L9" s="15" t="inlineStr"/>
+      <c r="H9" s="21" t="inlineStr"/>
+      <c r="I9" s="21" t="inlineStr"/>
+      <c r="J9" s="22" t="inlineStr"/>
+      <c r="K9" s="21" t="inlineStr"/>
+      <c r="L9" s="17" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="12" t="n">
+      <c r="A10" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>Peak United 2014</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>Peak United</t>
         </is>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="15" t="n">
         <v>71.59999999999999</v>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>CO #29</t>
         </is>
       </c>
-      <c r="F10" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="G10" s="13" t="inlineStr">
+      <c r="F10" s="16" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
         <is>
           <t>Tier 2</t>
         </is>
       </c>
-      <c r="H10" s="10" t="inlineStr"/>
-      <c r="I10" s="10" t="inlineStr"/>
-      <c r="J10" s="11" t="inlineStr"/>
-      <c r="K10" s="10" t="inlineStr"/>
+      <c r="H10" s="11" t="inlineStr"/>
+      <c r="I10" s="11" t="inlineStr"/>
+      <c r="J10" s="12" t="inlineStr"/>
+      <c r="K10" s="11" t="inlineStr"/>
       <c r="L10" s="7" t="inlineStr"/>
     </row>
     <row r="11" ht="30" customHeight="1">
@@ -1255,54 +1246,50 @@
           <t>CO #37</t>
         </is>
       </c>
-      <c r="F11" s="7" t="n">
-        <v>5</v>
-      </c>
+      <c r="F11" s="10" t="inlineStr"/>
       <c r="G11" s="8" t="inlineStr">
         <is>
           <t>Tier 2</t>
         </is>
       </c>
-      <c r="H11" s="10" t="inlineStr"/>
-      <c r="I11" s="10" t="inlineStr"/>
-      <c r="J11" s="11" t="inlineStr"/>
-      <c r="K11" s="10" t="inlineStr"/>
+      <c r="H11" s="11" t="inlineStr"/>
+      <c r="I11" s="11" t="inlineStr"/>
+      <c r="J11" s="12" t="inlineStr"/>
+      <c r="K11" s="11" t="inlineStr"/>
       <c r="L11" s="7" t="inlineStr"/>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="12" t="n">
+      <c r="A12" s="13" t="n">
         <v>6</v>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>Sample Select 2014</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>Sample Select</t>
         </is>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="15" t="n">
         <v>67.40000000000001</v>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="13" t="inlineStr">
         <is>
           <t>CO #42</t>
         </is>
       </c>
-      <c r="F12" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="G12" s="13" t="inlineStr">
+      <c r="F12" s="16" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
         <is>
           <t>Tier 2</t>
         </is>
       </c>
-      <c r="H12" s="10" t="inlineStr"/>
-      <c r="I12" s="10" t="inlineStr"/>
-      <c r="J12" s="11" t="inlineStr"/>
-      <c r="K12" s="10" t="inlineStr"/>
+      <c r="H12" s="11" t="inlineStr"/>
+      <c r="I12" s="11" t="inlineStr"/>
+      <c r="J12" s="12" t="inlineStr"/>
+      <c r="K12" s="11" t="inlineStr"/>
       <c r="L12" s="7" t="inlineStr"/>
     </row>
     <row r="13" ht="45" customHeight="1">
@@ -1325,16 +1312,16 @@
           <t>CO #50</t>
         </is>
       </c>
-      <c r="F13" s="7" t="n"/>
+      <c r="F13" s="10" t="inlineStr"/>
       <c r="G13" s="8" t="inlineStr">
         <is>
           <t>Data review required · Confirm the team identity before seeding.</t>
         </is>
       </c>
-      <c r="H13" s="10" t="inlineStr"/>
-      <c r="I13" s="10" t="inlineStr"/>
-      <c r="J13" s="11" t="inlineStr"/>
-      <c r="K13" s="10" t="inlineStr"/>
+      <c r="H13" s="11" t="inlineStr"/>
+      <c r="I13" s="11" t="inlineStr"/>
+      <c r="J13" s="12" t="inlineStr"/>
+      <c r="K13" s="11" t="inlineStr"/>
       <c r="L13" s="7" t="inlineStr"/>
     </row>
     <row r="15">
@@ -1345,28 +1332,28 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t>Tier 1 — 3 teams: Double round robin; 4 games each; 6 matches; repeat opponents possible</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t>Tier 2 — 3 teams: Double round robin; 4 games each; 6 matches; repeat opponents possible</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="20" t="inlineStr">
+      <c r="A18" s="23" t="inlineStr">
         <is>
           <t>Small tier: no equally practical, fully assessed split keeps every tier at least 4 teams, preserves the supported strength breaks, and passes the competitive limits.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="20" t="inlineStr">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>Sample data only. Strength markers are observations, not automatic divisions.</t>
         </is>

</xml_diff>

<commit_message>
Find MatchBalance strength bands from whole-group evidence
</commit_message>
<xml_diff>
--- a/docs/design/matchbalance-excel/director-workbook-sample.xlsx
+++ b/docs/design/matchbalance-excel/director-workbook-sample.xlsx
@@ -14,7 +14,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'U10 Boys'!$1:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$L$18</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'U12 Girls'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$L$19</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$L$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -157,6 +157,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -174,9 +177,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -768,38 +768,38 @@
       <c r="L8" s="7" t="inlineStr"/>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="17" t="n">
+      <c r="A9" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Desert United 2016</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Desert United</t>
         </is>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="9" t="n">
         <v>84.59999999999999</v>
       </c>
-      <c r="E9" s="17" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>AZ #11</t>
         </is>
       </c>
-      <c r="F9" s="20" t="inlineStr"/>
-      <c r="G9" s="18" t="inlineStr">
+      <c r="F9" s="10" t="inlineStr"/>
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>Tier 1 · Strength gap below</t>
         </is>
       </c>
-      <c r="H9" s="21" t="inlineStr"/>
-      <c r="I9" s="21" t="inlineStr"/>
-      <c r="J9" s="22" t="inlineStr"/>
-      <c r="K9" s="21" t="inlineStr"/>
-      <c r="L9" s="17" t="inlineStr"/>
+      <c r="H9" s="11" t="inlineStr"/>
+      <c r="I9" s="11" t="inlineStr"/>
+      <c r="J9" s="12" t="inlineStr"/>
+      <c r="K9" s="11" t="inlineStr"/>
+      <c r="L9" s="7" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="13" t="n">
@@ -903,28 +903,28 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>Tier 1 — 5 teams: Round robin; 4 games each; 10 matches</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="23" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Matchup review needed: this split still includes potentially uneven games.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="23" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Review this matchup: Juniper FC 2016 Blue vs Mesa Juniors 2016; projected goal gap 4.00, chance of a 4+ goal margin 55%.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="23" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Sample workbook: use the yellow columns for the director's final decisions.</t>
         </is>
@@ -973,7 +973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1156,38 +1156,38 @@
       <c r="L8" s="7" t="inlineStr"/>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="17" t="n">
+      <c r="A9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="18" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>Aspen Athletic 2014</t>
         </is>
       </c>
-      <c r="C9" s="18" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>Aspen Athletic</t>
         </is>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="20" t="n">
         <v>83.89999999999999</v>
       </c>
-      <c r="E9" s="17" t="inlineStr">
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>CO #15</t>
         </is>
       </c>
-      <c r="F9" s="20" t="inlineStr"/>
-      <c r="G9" s="18" t="inlineStr">
+      <c r="F9" s="21" t="inlineStr"/>
+      <c r="G9" s="19" t="inlineStr">
         <is>
           <t>Tier 1 · Strength gap below</t>
         </is>
       </c>
-      <c r="H9" s="21" t="inlineStr"/>
-      <c r="I9" s="21" t="inlineStr"/>
-      <c r="J9" s="22" t="inlineStr"/>
-      <c r="K9" s="21" t="inlineStr"/>
-      <c r="L9" s="17" t="inlineStr"/>
+      <c r="H9" s="22" t="inlineStr"/>
+      <c r="I9" s="22" t="inlineStr"/>
+      <c r="J9" s="23" t="inlineStr"/>
+      <c r="K9" s="22" t="inlineStr"/>
+      <c r="L9" s="18" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="13" t="n">
@@ -1332,35 +1332,43 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="23" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Tier 1 — 3 teams: Double round robin; 4 games each; 6 matches; repeat opponents possible</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="23" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Tier 2 — 3 teams: Double round robin; 4 games each; 6 matches; repeat opponents possible</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="23" t="inlineStr">
-        <is>
-          <t>Small tier: no equally practical, fully assessed split keeps every tier at least 4 teams, preserves the supported strength breaks, and passes the competitive limits.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="23" t="inlineStr">
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Tiers compare results across whole groups. Teams near a break may still be closely matched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Small tier: no equally practical, fully assessed split with fewer tiers below 4 teams passes the competitive limits. Review the teams near this break.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Sample data only. Strength markers are observations, not automatic divisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
+    <mergeCell ref="A20:L20"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A16:L16"/>
     <mergeCell ref="A19:L19"/>

</xml_diff>

<commit_message>
Use game evidence for MatchBalance seed order and practical tier guidance (#1333)
* Use game evidence for MatchBalance seed order and practical tier guidance

* Keep MatchBalance scoring rates within connected game evidence

* Simplify MatchBalance director sheets while preserving review warnings

* Restore MatchBalance sheet details and yellow competitive breaks

* Choose practical MatchBalance tiers without overriding safe game evidence

* Show national cohort ranks instead of seed changes on director sheets

* Find MatchBalance strength bands from whole-group evidence

* Simplify MatchBalance review and default new runs to game evidence
</commit_message>
<xml_diff>
--- a/docs/design/matchbalance-excel/director-workbook-sample.xlsx
+++ b/docs/design/matchbalance-excel/director-workbook-sample.xlsx
@@ -12,9 +12,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'U10 Boys'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$K$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$L$18</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'U12 Girls'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$K$21</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$L$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -111,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -136,6 +136,9 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -151,6 +154,12 @@
     <xf numFmtId="164" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -160,14 +169,14 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -246,40 +255,42 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Cohort1" displayName="Cohort1" ref="A6:K12" headerRowCount="1">
-  <autoFilter ref="A6:K12"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Cohort1" displayName="Cohort1" ref="A6:L12" headerRowCount="1">
+  <autoFilter ref="A6:L12"/>
+  <tableColumns count="12">
     <tableColumn id="1" name="MatchBalance seed"/>
     <tableColumn id="2" name="Team name"/>
     <tableColumn id="3" name="Club"/>
     <tableColumn id="4" name="PowerScore"/>
     <tableColumn id="5" name="State rank"/>
-    <tableColumn id="6" name="PowerScore seed"/>
-    <tableColumn id="7" name="Movement / placement notes"/>
+    <tableColumn id="6" name="National rank"/>
+    <tableColumn id="7" name="Tier / placement"/>
     <tableColumn id="8" name="Final division"/>
     <tableColumn id="9" name="Pool"/>
     <tableColumn id="10" name="Final seed"/>
     <tableColumn id="11" name="Director notes"/>
+    <tableColumn id="12" name="Record (W-L-D)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Cohort2" displayName="Cohort2" ref="A6:K13" headerRowCount="1">
-  <autoFilter ref="A6:K13"/>
-  <tableColumns count="11">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Cohort2" displayName="Cohort2" ref="A6:L13" headerRowCount="1">
+  <autoFilter ref="A6:L13"/>
+  <tableColumns count="12">
     <tableColumn id="1" name="MatchBalance seed"/>
     <tableColumn id="2" name="Team name"/>
     <tableColumn id="3" name="Club"/>
     <tableColumn id="4" name="PowerScore"/>
     <tableColumn id="5" name="State rank"/>
-    <tableColumn id="6" name="PowerScore seed"/>
-    <tableColumn id="7" name="Movement / placement notes"/>
+    <tableColumn id="6" name="National rank"/>
+    <tableColumn id="7" name="Tier / placement"/>
     <tableColumn id="8" name="Final division"/>
     <tableColumn id="9" name="Pool"/>
     <tableColumn id="10" name="Final seed"/>
     <tableColumn id="11" name="Director notes"/>
+    <tableColumn id="12" name="Record (W-L-D)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -574,7 +585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -588,6 +599,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -607,7 +619,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark boundaries where nearby projected matchups meaningfully worsen; the PowerScore difference is supporting context; they do not assign divisions or pools. Recommended tier breaks use practical division sizes and all potential matchups. A tier can contain multiple pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
+          <t>Read from seed 1 down. Tier lines suggest strength divisions; a division can contain several pools. Natural separation marks a strength gap; practical splits also consider usable division sizes. Review warnings and unplaced teams before making final placements.</t>
         </is>
       </c>
     </row>
@@ -653,12 +665,12 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>PowerScore seed</t>
+          <t>National rank</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Movement / placement notes</t>
+          <t>Tier / placement</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -679,6 +691,11 @@
       <c r="K6" s="6" t="inlineStr">
         <is>
           <t>Director notes</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>Record (W-L-D)</t>
         </is>
       </c>
     </row>
@@ -704,125 +721,121 @@
           <t>AZ #2</t>
         </is>
       </c>
-      <c r="F7" s="7" t="n">
-        <v>1</v>
-      </c>
+      <c r="F7" s="10" t="inlineStr"/>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>Tier 1 · Seeded</t>
-        </is>
-      </c>
-      <c r="H7" s="10" t="inlineStr"/>
-      <c r="I7" s="10" t="inlineStr"/>
-      <c r="J7" s="11" t="inlineStr"/>
-      <c r="K7" s="10" t="inlineStr"/>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr"/>
+      <c r="I7" s="11" t="inlineStr"/>
+      <c r="J7" s="12" t="inlineStr"/>
+      <c r="K7" s="11" t="inlineStr"/>
+      <c r="L7" s="7" t="inlineStr"/>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>Copper State 2016</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>Copper State</t>
         </is>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="15" t="n">
         <v>87.2</v>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>AZ #6</t>
         </is>
       </c>
-      <c r="F8" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="G8" s="13" t="inlineStr">
-        <is>
-          <t>Tier 1 · Seeded</t>
-        </is>
-      </c>
-      <c r="H8" s="10" t="inlineStr"/>
-      <c r="I8" s="10" t="inlineStr"/>
-      <c r="J8" s="11" t="inlineStr"/>
-      <c r="K8" s="10" t="inlineStr"/>
-    </row>
-    <row r="9" ht="105" customHeight="1">
-      <c r="A9" s="15" t="n">
+      <c r="F8" s="16" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="inlineStr"/>
+      <c r="I8" s="11" t="inlineStr"/>
+      <c r="J8" s="12" t="inlineStr"/>
+      <c r="K8" s="11" t="inlineStr"/>
+      <c r="L8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
         <is>
           <t>Desert United 2016</t>
         </is>
       </c>
-      <c r="C9" s="16" t="inlineStr">
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>Desert United</t>
         </is>
       </c>
-      <c r="D9" s="17" t="n">
+      <c r="D9" s="9" t="n">
         <v>84.59999999999999</v>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>AZ #11</t>
         </is>
       </c>
-      <c r="F9" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="G9" s="16" t="inlineStr">
-        <is>
-          <t>Tier 1 · Competitive Break: projected matchup quality worsens between seeds 3 and 4; PowerScore difference 11.7 points. · Competitive Break: natural strength separation · Very close: seeds 1-3 · Seeded</t>
-        </is>
-      </c>
-      <c r="H9" s="18" t="inlineStr"/>
-      <c r="I9" s="18" t="inlineStr"/>
-      <c r="J9" s="19" t="inlineStr"/>
-      <c r="K9" s="18" t="inlineStr"/>
+      <c r="F9" s="10" t="inlineStr"/>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>Tier 1 · Strength gap below</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr"/>
+      <c r="I9" s="11" t="inlineStr"/>
+      <c r="J9" s="12" t="inlineStr"/>
+      <c r="K9" s="11" t="inlineStr"/>
+      <c r="L9" s="7" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="12" t="n">
+      <c r="A10" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>Valley Athletic 2016</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>Valley Athletic</t>
         </is>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="15" t="n">
         <v>72.89999999999999</v>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>AZ #24</t>
         </is>
       </c>
-      <c r="F10" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>Tier 1 · Seeded</t>
-        </is>
-      </c>
-      <c r="H10" s="10" t="inlineStr"/>
-      <c r="I10" s="10" t="inlineStr"/>
-      <c r="J10" s="11" t="inlineStr"/>
-      <c r="K10" s="10" t="inlineStr"/>
-    </row>
-    <row r="11" ht="30" customHeight="1">
+      <c r="F10" s="16" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr"/>
+      <c r="I10" s="11" t="inlineStr"/>
+      <c r="J10" s="12" t="inlineStr"/>
+      <c r="K10" s="11" t="inlineStr"/>
+      <c r="L10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11" ht="15" customHeight="1">
       <c r="A11" s="7" t="n">
         <v>5</v>
       </c>
@@ -844,43 +857,43 @@
           <t>AZ #32</t>
         </is>
       </c>
-      <c r="F11" s="7" t="n">
-        <v>5</v>
-      </c>
+      <c r="F11" s="10" t="inlineStr"/>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>Tier 1 · Very close: seeds 4-5 · Seeded</t>
-        </is>
-      </c>
-      <c r="H11" s="10" t="inlineStr"/>
-      <c r="I11" s="10" t="inlineStr"/>
-      <c r="J11" s="11" t="inlineStr"/>
-      <c r="K11" s="10" t="inlineStr"/>
-    </row>
-    <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="12" t="n"/>
-      <c r="B12" s="13" t="inlineStr">
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="inlineStr"/>
+      <c r="I11" s="11" t="inlineStr"/>
+      <c r="J11" s="12" t="inlineStr"/>
+      <c r="K11" s="11" t="inlineStr"/>
+      <c r="L11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="13" t="n"/>
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>Sample Academy 2016</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>Sample Academy</t>
         </is>
       </c>
-      <c r="D12" s="12" t="n"/>
-      <c r="E12" s="12" t="inlineStr"/>
-      <c r="F12" s="12" t="n"/>
-      <c r="G12" s="13" t="inlineStr">
-        <is>
-          <t>Not found in PitchRank</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr"/>
-      <c r="I12" s="10" t="inlineStr"/>
-      <c r="J12" s="11" t="inlineStr"/>
-      <c r="K12" s="10" t="inlineStr"/>
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="13" t="inlineStr"/>
+      <c r="F12" s="16" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>Not found in PitchRank · Not found in PitchRank.</t>
+        </is>
+      </c>
+      <c r="H12" s="11" t="inlineStr"/>
+      <c r="I12" s="11" t="inlineStr"/>
+      <c r="J12" s="12" t="inlineStr"/>
+      <c r="K12" s="11" t="inlineStr"/>
+      <c r="L12" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -889,61 +902,45 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="20" t="inlineStr">
-        <is>
-          <t>Tier 1: seeds 1-5 (5 teams; Partial round robin; 3 guaranteed; up to 4 games; 8 matches total; no playoffs; Use points per game for unequal preliminary game counts; all played games still count toward the game guarantee.; compatible pools 5)</t>
+    <row r="15" ht="15" customHeight="1">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>Tier 1 — 5 teams: Round robin; 4 games each; 10 matches</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="20" t="inlineStr">
-        <is>
-          <t>5 of 6 teams assessed in the tier order; 1 still need placement. These breaks cover the assessed subset.</t>
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Matchup review needed: this split still includes potentially uneven games.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="20" t="inlineStr">
-        <is>
-          <t>Review-required compromise: every evaluated arrangement retains projected mismatches.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="20" t="inlineStr">
-        <is>
-          <t>Worst remaining mismatch: Juniper FC 2016 Blue vs Mesa Juniors 2016; expected absolute goal difference 4.00, four-goal margin probability 55%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="20" t="inlineStr">
-        <is>
-          <t>Formats use the saved MatchBalance profile; confirm game guarantees and event logistics.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="20" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Review this matchup: Juniper FC 2016 Blue vs Mesa Juniors 2016; projected goal gap 4.00, chance of a 4+ goal margin 55%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Sample workbook: use the yellow columns for the director's final decisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A18:K18"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A20:K20"/>
-    <mergeCell ref="A15:K15"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A16:K16"/>
-    <mergeCell ref="A19:K19"/>
-    <mergeCell ref="A5:K5"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A17:K17"/>
+  <mergeCells count="9">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A16:L16"/>
+    <mergeCell ref="A15:L15"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A17:L17"/>
+    <mergeCell ref="A18:L18"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A4:L4"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D11">
     <cfRule type="dataBar" priority="1">
@@ -976,7 +973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -990,6 +987,7 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1009,7 +1007,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Start with the numbered MatchBalance Seed order. PowerScore remains the original published-strength baseline; bars use the same 0-100 scale. Competitive Breaks mark boundaries where nearby projected matchups meaningfully worsen; the PowerScore difference is supporting context; they do not assign divisions or pools. Recommended tier breaks use practical division sizes and all potential matchups. A tier can contain multiple pools. Very-close ranges identify the same competitive neighborhood without claiming the teams are equal.</t>
+          <t>Read from seed 1 down. Tier lines suggest strength divisions; a division can contain several pools. Natural separation marks a strength gap; practical splits also consider usable division sizes. Review warnings and unplaced teams before making final placements.</t>
         </is>
       </c>
     </row>
@@ -1055,12 +1053,12 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>PowerScore seed</t>
+          <t>National rank</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
         <is>
-          <t>Movement / placement notes</t>
+          <t>Tier / placement</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr">
@@ -1081,6 +1079,11 @@
       <c r="K6" s="6" t="inlineStr">
         <is>
           <t>Director notes</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>Record (W-L-D)</t>
         </is>
       </c>
     </row>
@@ -1106,123 +1109,119 @@
           <t>CO #4</t>
         </is>
       </c>
-      <c r="F7" s="7" t="n">
-        <v>1</v>
-      </c>
+      <c r="F7" s="10" t="inlineStr"/>
       <c r="G7" s="8" t="inlineStr">
         <is>
-          <t>Tier 1 · Seeded</t>
-        </is>
-      </c>
-      <c r="H7" s="10" t="inlineStr"/>
-      <c r="I7" s="10" t="inlineStr"/>
-      <c r="J7" s="11" t="inlineStr"/>
-      <c r="K7" s="10" t="inlineStr"/>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr"/>
+      <c r="I7" s="11" t="inlineStr"/>
+      <c r="J7" s="12" t="inlineStr"/>
+      <c r="K7" s="11" t="inlineStr"/>
+      <c r="L7" s="7" t="inlineStr"/>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>Front Range FC 2014</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>Front Range FC</t>
         </is>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="15" t="n">
         <v>86.5</v>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>CO #9</t>
         </is>
       </c>
-      <c r="F8" s="12" t="n">
-        <v>2</v>
-      </c>
-      <c r="G8" s="13" t="inlineStr">
-        <is>
-          <t>Tier 1 · Seeded</t>
-        </is>
-      </c>
-      <c r="H8" s="10" t="inlineStr"/>
-      <c r="I8" s="10" t="inlineStr"/>
-      <c r="J8" s="11" t="inlineStr"/>
-      <c r="K8" s="10" t="inlineStr"/>
-    </row>
-    <row r="9" ht="105" customHeight="1">
-      <c r="A9" s="15" t="n">
+      <c r="F8" s="16" t="inlineStr"/>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>Tier 1</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="inlineStr"/>
+      <c r="I8" s="11" t="inlineStr"/>
+      <c r="J8" s="12" t="inlineStr"/>
+      <c r="K8" s="11" t="inlineStr"/>
+      <c r="L8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="19" t="inlineStr">
         <is>
           <t>Aspen Athletic 2014</t>
         </is>
       </c>
-      <c r="C9" s="16" t="inlineStr">
+      <c r="C9" s="19" t="inlineStr">
         <is>
           <t>Aspen Athletic</t>
         </is>
       </c>
-      <c r="D9" s="17" t="n">
+      <c r="D9" s="20" t="n">
         <v>83.89999999999999</v>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="E9" s="18" t="inlineStr">
         <is>
           <t>CO #15</t>
         </is>
       </c>
-      <c r="F9" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="G9" s="16" t="inlineStr">
-        <is>
-          <t>Tier 1 · Competitive Break: projected matchup quality worsens between seeds 3 and 4; PowerScore difference 12.3 points. · Recommended tier break + natural strength separation · Very close: seeds 1-3 · Seeded</t>
-        </is>
-      </c>
-      <c r="H9" s="18" t="inlineStr"/>
-      <c r="I9" s="18" t="inlineStr"/>
-      <c r="J9" s="19" t="inlineStr"/>
-      <c r="K9" s="18" t="inlineStr"/>
+      <c r="F9" s="21" t="inlineStr"/>
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>Tier 1 · Strength gap below</t>
+        </is>
+      </c>
+      <c r="H9" s="22" t="inlineStr"/>
+      <c r="I9" s="22" t="inlineStr"/>
+      <c r="J9" s="23" t="inlineStr"/>
+      <c r="K9" s="22" t="inlineStr"/>
+      <c r="L9" s="18" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="12" t="n">
+      <c r="A10" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>Peak United 2014</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>Peak United</t>
         </is>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="15" t="n">
         <v>71.59999999999999</v>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>CO #29</t>
         </is>
       </c>
-      <c r="F10" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="G10" s="13" t="inlineStr">
-        <is>
-          <t>Tier 2 · Seeded</t>
-        </is>
-      </c>
-      <c r="H10" s="10" t="inlineStr"/>
-      <c r="I10" s="10" t="inlineStr"/>
-      <c r="J10" s="11" t="inlineStr"/>
-      <c r="K10" s="10" t="inlineStr"/>
+      <c r="F10" s="16" t="inlineStr"/>
+      <c r="G10" s="14" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr"/>
+      <c r="I10" s="11" t="inlineStr"/>
+      <c r="J10" s="12" t="inlineStr"/>
+      <c r="K10" s="11" t="inlineStr"/>
+      <c r="L10" s="7" t="inlineStr"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="7" t="n">
@@ -1247,55 +1246,53 @@
           <t>CO #37</t>
         </is>
       </c>
-      <c r="F11" s="7" t="n">
-        <v>5</v>
-      </c>
+      <c r="F11" s="10" t="inlineStr"/>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>Tier 2 · Seeded</t>
-        </is>
-      </c>
-      <c r="H11" s="10" t="inlineStr"/>
-      <c r="I11" s="10" t="inlineStr"/>
-      <c r="J11" s="11" t="inlineStr"/>
-      <c r="K11" s="10" t="inlineStr"/>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="12" t="n">
+          <t>Tier 2</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="inlineStr"/>
+      <c r="I11" s="11" t="inlineStr"/>
+      <c r="J11" s="12" t="inlineStr"/>
+      <c r="K11" s="11" t="inlineStr"/>
+      <c r="L11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="13" t="n">
         <v>6</v>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>Sample Select 2014</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>Sample Select</t>
         </is>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="15" t="n">
         <v>67.40000000000001</v>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="13" t="inlineStr">
         <is>
           <t>CO #42</t>
         </is>
       </c>
-      <c r="F12" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="G12" s="13" t="inlineStr">
-        <is>
-          <t>Tier 2 · Very close: seeds 4-6 · Seeded</t>
-        </is>
-      </c>
-      <c r="H12" s="10" t="inlineStr"/>
-      <c r="I12" s="10" t="inlineStr"/>
-      <c r="J12" s="11" t="inlineStr"/>
-      <c r="K12" s="10" t="inlineStr"/>
-    </row>
-    <row r="13" ht="15" customHeight="1">
+      <c r="F12" s="16" t="inlineStr"/>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>Tier 2</t>
+        </is>
+      </c>
+      <c r="H12" s="11" t="inlineStr"/>
+      <c r="I12" s="11" t="inlineStr"/>
+      <c r="J12" s="12" t="inlineStr"/>
+      <c r="K12" s="11" t="inlineStr"/>
+      <c r="L12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13" ht="45" customHeight="1">
       <c r="A13" s="7" t="n"/>
       <c r="B13" s="8" t="inlineStr">
         <is>
@@ -1315,16 +1312,17 @@
           <t>CO #50</t>
         </is>
       </c>
-      <c r="F13" s="7" t="n"/>
+      <c r="F13" s="10" t="inlineStr"/>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>Data review required</t>
-        </is>
-      </c>
-      <c r="H13" s="10" t="inlineStr"/>
-      <c r="I13" s="10" t="inlineStr"/>
-      <c r="J13" s="11" t="inlineStr"/>
-      <c r="K13" s="10" t="inlineStr"/>
+          <t>Data review required · Confirm the team identity before seeding.</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="inlineStr"/>
+      <c r="I13" s="11" t="inlineStr"/>
+      <c r="J13" s="12" t="inlineStr"/>
+      <c r="K13" s="11" t="inlineStr"/>
+      <c r="L13" s="7" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1333,61 +1331,53 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="20" t="inlineStr">
-        <is>
-          <t>Tier 1: seeds 1-3 (3 teams; Round robin, extra points match and final; 3 guaranteed; up to 4 games; 5 matches total; opponents may meet up to 2 times; includes playoffs; compatible pools 3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="30" customHeight="1">
-      <c r="A17" s="20" t="inlineStr">
-        <is>
-          <t>Tier 2: seeds 4-6 (3 teams; Round robin, extra points match and final; 3 guaranteed; up to 4 games; 5 matches total; opponents may meet up to 2 times; includes playoffs; compatible pools 3)</t>
+    <row r="16" ht="15" customHeight="1">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>Tier 1 — 3 teams: Double round robin; 4 games each; 6 matches; repeat opponents possible</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="15" customHeight="1">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>Tier 2 — 3 teams: Double round robin; 4 games each; 6 matches; repeat opponents possible</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="20" t="inlineStr">
-        <is>
-          <t>6 of 7 teams assessed in the tier order; 1 still need placement. These breaks cover the assessed subset.</t>
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>Tiers compare results across whole groups. Teams near a break may still be closely matched.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="20" t="inlineStr">
-        <is>
-          <t>Small-division fallback: no complete, fully assessed arrangement with every strength division at least 4 teams passes the competitive limits and format restrictions. Smaller pools inside a larger strength division are still allowed.</t>
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Small tier: no equally practical, fully assessed split with fewer tiers below 4 teams passes the competitive limits. Review the teams near this break.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="20" t="inlineStr">
-        <is>
-          <t>Formats use the saved MatchBalance profile; confirm game guarantees and event logistics.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="20" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Sample data only. Strength markers are observations, not automatic divisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A18:K18"/>
-    <mergeCell ref="A4:K4"/>
-    <mergeCell ref="A3:K3"/>
-    <mergeCell ref="A20:K20"/>
-    <mergeCell ref="A21:K21"/>
-    <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A16:K16"/>
-    <mergeCell ref="A19:K19"/>
-    <mergeCell ref="A5:K5"/>
-    <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A17:K17"/>
+  <mergeCells count="10">
+    <mergeCell ref="A20:L20"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A16:L16"/>
+    <mergeCell ref="A19:L19"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A5:L5"/>
+    <mergeCell ref="A17:L17"/>
+    <mergeCell ref="A18:L18"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="A4:L4"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D12">
     <cfRule type="dataBar" priority="1">

</xml_diff>

<commit_message>
Refresh matched teams automatically and simplify director reports
</commit_message>
<xml_diff>
--- a/docs/design/matchbalance-excel/director-workbook-sample.xlsx
+++ b/docs/design/matchbalance-excel/director-workbook-sample.xlsx
@@ -12,9 +12,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'U10 Boys'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$L$18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$L$17</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'U12 Girls'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$L$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$L$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,10 +42,6 @@
     <font>
       <b val="1"/>
       <color rgb="00083E33"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="005B6B66"/>
     </font>
     <font>
       <color rgb="005B6B66"/>
@@ -111,20 +107,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -585,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -616,330 +609,315 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Read from seed 1 down. Tier lines suggest strength divisions; a division can contain several pools. Natural separation marks a strength gap; practical splits also consider usable division sizes. Review warnings and unplaced teams before making final placements.</t>
-        </is>
-      </c>
-    </row>
+    <row r="3" ht="6" customHeight="1"/>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Ratings as of 2026-09-22 · Generated 2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Review-required compromise: 5 teams. Seeded: 5 · Not found in PitchRank: 1 · No current rating: 0 · Data review required: 0</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>5 teams ranked · 1 need placement. Matchup review needed before finalizing</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>MatchBalance seed</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Team name</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Club</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>PowerScore</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>State rank</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>National rank</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Tier / placement</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Final division</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>Pool</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>Final seed</t>
         </is>
       </c>
-      <c r="K6" s="6" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>Director notes</t>
         </is>
       </c>
-      <c r="L6" s="6" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
         <is>
           <t>Record (W-L-D)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Juniper FC 2016 Blue</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Juniper FC</t>
         </is>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="8" t="n">
         <v>90.10000000000001</v>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>AZ #2</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr"/>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="H7" s="11" t="inlineStr"/>
-      <c r="I7" s="11" t="inlineStr"/>
-      <c r="J7" s="12" t="inlineStr"/>
-      <c r="K7" s="11" t="inlineStr"/>
-      <c r="L7" s="7" t="inlineStr"/>
+      <c r="H7" s="10" t="inlineStr"/>
+      <c r="I7" s="10" t="inlineStr"/>
+      <c r="J7" s="11" t="inlineStr"/>
+      <c r="K7" s="10" t="inlineStr"/>
+      <c r="L7" s="6" t="inlineStr"/>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="13" t="n">
+      <c r="A8" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Copper State 2016</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>Copper State</t>
         </is>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="14" t="n">
         <v>87.2</v>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>AZ #6</t>
         </is>
       </c>
-      <c r="F8" s="16" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
+      <c r="F8" s="15" t="inlineStr"/>
+      <c r="G8" s="13" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="H8" s="11" t="inlineStr"/>
-      <c r="I8" s="11" t="inlineStr"/>
-      <c r="J8" s="12" t="inlineStr"/>
-      <c r="K8" s="11" t="inlineStr"/>
-      <c r="L8" s="7" t="inlineStr"/>
+      <c r="H8" s="10" t="inlineStr"/>
+      <c r="I8" s="10" t="inlineStr"/>
+      <c r="J8" s="11" t="inlineStr"/>
+      <c r="K8" s="10" t="inlineStr"/>
+      <c r="L8" s="6" t="inlineStr"/>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Desert United 2016</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Desert United</t>
         </is>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="8" t="n">
         <v>84.59999999999999</v>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>AZ #11</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr"/>
-      <c r="G9" s="8" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr"/>
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>Tier 1 · Strength gap below</t>
         </is>
       </c>
-      <c r="H9" s="11" t="inlineStr"/>
-      <c r="I9" s="11" t="inlineStr"/>
-      <c r="J9" s="12" t="inlineStr"/>
-      <c r="K9" s="11" t="inlineStr"/>
-      <c r="L9" s="7" t="inlineStr"/>
+      <c r="H9" s="10" t="inlineStr"/>
+      <c r="I9" s="10" t="inlineStr"/>
+      <c r="J9" s="11" t="inlineStr"/>
+      <c r="K9" s="10" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="13" t="n">
+      <c r="A10" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Valley Athletic 2016</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>Valley Athletic</t>
         </is>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="14" t="n">
         <v>72.89999999999999</v>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>AZ #24</t>
         </is>
       </c>
-      <c r="F10" s="16" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
+      <c r="F10" s="15" t="inlineStr"/>
+      <c r="G10" s="13" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="H10" s="11" t="inlineStr"/>
-      <c r="I10" s="11" t="inlineStr"/>
-      <c r="J10" s="12" t="inlineStr"/>
-      <c r="K10" s="11" t="inlineStr"/>
-      <c r="L10" s="7" t="inlineStr"/>
+      <c r="H10" s="10" t="inlineStr"/>
+      <c r="I10" s="10" t="inlineStr"/>
+      <c r="J10" s="11" t="inlineStr"/>
+      <c r="K10" s="10" t="inlineStr"/>
+      <c r="L10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Mesa Juniors 2016</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Mesa Juniors</t>
         </is>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="8" t="n">
         <v>70.09999999999999</v>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>AZ #32</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr"/>
-      <c r="G11" s="8" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr"/>
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="H11" s="11" t="inlineStr"/>
-      <c r="I11" s="11" t="inlineStr"/>
-      <c r="J11" s="12" t="inlineStr"/>
-      <c r="K11" s="11" t="inlineStr"/>
-      <c r="L11" s="7" t="inlineStr"/>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="13" t="n"/>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="H11" s="10" t="inlineStr"/>
+      <c r="I11" s="10" t="inlineStr"/>
+      <c r="J11" s="11" t="inlineStr"/>
+      <c r="K11" s="10" t="inlineStr"/>
+      <c r="L11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Sample Academy 2016</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>Sample Academy</t>
         </is>
       </c>
-      <c r="D12" s="13" t="n"/>
-      <c r="E12" s="13" t="inlineStr"/>
-      <c r="F12" s="16" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>Not found in PitchRank · Not found in PitchRank.</t>
-        </is>
-      </c>
-      <c r="H12" s="11" t="inlineStr"/>
-      <c r="I12" s="11" t="inlineStr"/>
-      <c r="J12" s="12" t="inlineStr"/>
-      <c r="K12" s="11" t="inlineStr"/>
-      <c r="L12" s="7" t="inlineStr"/>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="12" t="inlineStr"/>
+      <c r="F12" s="15" t="inlineStr"/>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>Not found in PitchRank.</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr"/>
+      <c r="I12" s="10" t="inlineStr"/>
+      <c r="J12" s="11" t="inlineStr"/>
+      <c r="K12" s="10" t="inlineStr"/>
+      <c r="L12" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Director notes</t>
+          <t>Teams to review</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="17" t="inlineStr">
-        <is>
-          <t>Tier 1 — 5 teams: Round robin; 4 games each; 10 matches</t>
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Matchup review needed: this split still includes potentially uneven games.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>Matchup review needed: this split still includes potentially uneven games.</t>
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Review this matchup: Juniper FC 2016 Blue vs Mesa Juniors 2016; projected goal gap 4.00, chance of a 4+ goal margin 55%.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>Review this matchup: Juniper FC 2016 Blue vs Mesa Juniors 2016; projected goal gap 4.00, chance of a 4+ goal margin 55%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>Sample workbook: use the yellow columns for the director's final decisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="7">
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A16:L16"/>
     <mergeCell ref="A15:L15"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A5:L5"/>
     <mergeCell ref="A17:L17"/>
-    <mergeCell ref="A18:L18"/>
-    <mergeCell ref="A3:L3"/>
     <mergeCell ref="A4:L4"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D11">
@@ -973,7 +951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1004,379 +982,348 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Read from seed 1 down. Tier lines suggest strength divisions; a division can contain several pools. Natural separation marks a strength gap; practical splits also consider usable division sizes. Review warnings and unplaced teams before making final placements.</t>
-        </is>
-      </c>
-    </row>
+    <row r="3" ht="6" customHeight="1"/>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Ratings as of 2026-09-22 · Generated 2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Suggested tiers: 3 + 3 teams. Seeded: 6 · Not found in PitchRank: 0 · No current rating: 0 · Data review required: 1</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>6 teams ranked · 1 need placement</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>MatchBalance seed</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Team name</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Club</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>PowerScore</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>State rank</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>National rank</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Tier / placement</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Final division</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>Pool</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>Final seed</t>
         </is>
       </c>
-      <c r="K6" s="6" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>Director notes</t>
         </is>
       </c>
-      <c r="L6" s="6" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
         <is>
           <t>Record (W-L-D)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Summit SC 2014 Green</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Summit SC</t>
         </is>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="8" t="n">
         <v>89.3</v>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>CO #4</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr"/>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="H7" s="11" t="inlineStr"/>
-      <c r="I7" s="11" t="inlineStr"/>
-      <c r="J7" s="12" t="inlineStr"/>
-      <c r="K7" s="11" t="inlineStr"/>
-      <c r="L7" s="7" t="inlineStr"/>
+      <c r="H7" s="10" t="inlineStr"/>
+      <c r="I7" s="10" t="inlineStr"/>
+      <c r="J7" s="11" t="inlineStr"/>
+      <c r="K7" s="10" t="inlineStr"/>
+      <c r="L7" s="6" t="inlineStr"/>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="13" t="n">
+      <c r="A8" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Front Range FC 2014</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>Front Range FC</t>
         </is>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="14" t="n">
         <v>86.5</v>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>CO #9</t>
         </is>
       </c>
-      <c r="F8" s="16" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
+      <c r="F8" s="15" t="inlineStr"/>
+      <c r="G8" s="13" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="H8" s="11" t="inlineStr"/>
-      <c r="I8" s="11" t="inlineStr"/>
-      <c r="J8" s="12" t="inlineStr"/>
-      <c r="K8" s="11" t="inlineStr"/>
-      <c r="L8" s="7" t="inlineStr"/>
+      <c r="H8" s="10" t="inlineStr"/>
+      <c r="I8" s="10" t="inlineStr"/>
+      <c r="J8" s="11" t="inlineStr"/>
+      <c r="K8" s="10" t="inlineStr"/>
+      <c r="L8" s="6" t="inlineStr"/>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="18" t="n">
+      <c r="A9" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>Aspen Athletic 2014</t>
         </is>
       </c>
-      <c r="C9" s="19" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>Aspen Athletic</t>
         </is>
       </c>
-      <c r="D9" s="20" t="n">
+      <c r="D9" s="19" t="n">
         <v>83.89999999999999</v>
       </c>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>CO #15</t>
         </is>
       </c>
-      <c r="F9" s="21" t="inlineStr"/>
-      <c r="G9" s="19" t="inlineStr">
+      <c r="F9" s="20" t="inlineStr"/>
+      <c r="G9" s="18" t="inlineStr">
         <is>
           <t>Tier 1 · Strength gap below</t>
         </is>
       </c>
-      <c r="H9" s="22" t="inlineStr"/>
-      <c r="I9" s="22" t="inlineStr"/>
-      <c r="J9" s="23" t="inlineStr"/>
-      <c r="K9" s="22" t="inlineStr"/>
-      <c r="L9" s="18" t="inlineStr"/>
+      <c r="H9" s="21" t="inlineStr"/>
+      <c r="I9" s="21" t="inlineStr"/>
+      <c r="J9" s="22" t="inlineStr"/>
+      <c r="K9" s="21" t="inlineStr"/>
+      <c r="L9" s="17" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="13" t="n">
+      <c r="A10" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Peak United 2014</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>Peak United</t>
         </is>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="14" t="n">
         <v>71.59999999999999</v>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>CO #29</t>
         </is>
       </c>
-      <c r="F10" s="16" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
+      <c r="F10" s="15" t="inlineStr"/>
+      <c r="G10" s="13" t="inlineStr">
         <is>
           <t>Tier 2</t>
         </is>
       </c>
-      <c r="H10" s="11" t="inlineStr"/>
-      <c r="I10" s="11" t="inlineStr"/>
-      <c r="J10" s="12" t="inlineStr"/>
-      <c r="K10" s="11" t="inlineStr"/>
-      <c r="L10" s="7" t="inlineStr"/>
+      <c r="H10" s="10" t="inlineStr"/>
+      <c r="I10" s="10" t="inlineStr"/>
+      <c r="J10" s="11" t="inlineStr"/>
+      <c r="K10" s="10" t="inlineStr"/>
+      <c r="L10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Foothills FC 2014
 Listed: Premier</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Foothills FC</t>
         </is>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="8" t="n">
         <v>68.89999999999999</v>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>CO #37</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr"/>
-      <c r="G11" s="8" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr"/>
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Tier 2</t>
         </is>
       </c>
-      <c r="H11" s="11" t="inlineStr"/>
-      <c r="I11" s="11" t="inlineStr"/>
-      <c r="J11" s="12" t="inlineStr"/>
-      <c r="K11" s="11" t="inlineStr"/>
-      <c r="L11" s="7" t="inlineStr"/>
+      <c r="H11" s="10" t="inlineStr"/>
+      <c r="I11" s="10" t="inlineStr"/>
+      <c r="J11" s="11" t="inlineStr"/>
+      <c r="K11" s="10" t="inlineStr"/>
+      <c r="L11" s="6" t="inlineStr"/>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="13" t="n">
+      <c r="A12" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Sample Select 2014</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>Sample Select</t>
         </is>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D12" s="14" t="n">
         <v>67.40000000000001</v>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="E12" s="12" t="inlineStr">
         <is>
           <t>CO #42</t>
         </is>
       </c>
-      <c r="F12" s="16" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
+      <c r="F12" s="15" t="inlineStr"/>
+      <c r="G12" s="13" t="inlineStr">
         <is>
           <t>Tier 2</t>
         </is>
       </c>
-      <c r="H12" s="11" t="inlineStr"/>
-      <c r="I12" s="11" t="inlineStr"/>
-      <c r="J12" s="12" t="inlineStr"/>
-      <c r="K12" s="11" t="inlineStr"/>
-      <c r="L12" s="7" t="inlineStr"/>
+      <c r="H12" s="10" t="inlineStr"/>
+      <c r="I12" s="10" t="inlineStr"/>
+      <c r="J12" s="11" t="inlineStr"/>
+      <c r="K12" s="10" t="inlineStr"/>
+      <c r="L12" s="6" t="inlineStr"/>
     </row>
     <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Review United 2014</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Review United</t>
         </is>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="8" t="n">
         <v>65</v>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>CO #50</t>
         </is>
       </c>
-      <c r="F13" s="10" t="inlineStr"/>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>Data review required · Confirm the team identity before seeding.</t>
-        </is>
-      </c>
-      <c r="H13" s="11" t="inlineStr"/>
-      <c r="I13" s="11" t="inlineStr"/>
-      <c r="J13" s="12" t="inlineStr"/>
-      <c r="K13" s="11" t="inlineStr"/>
-      <c r="L13" s="7" t="inlineStr"/>
+      <c r="F13" s="9" t="inlineStr"/>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Team data needs review. Confirm the team identity before seeding.</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr"/>
+      <c r="I13" s="10" t="inlineStr"/>
+      <c r="J13" s="11" t="inlineStr"/>
+      <c r="K13" s="10" t="inlineStr"/>
+      <c r="L13" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Director notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>Tier 1 — 3 teams: Double round robin; 4 games each; 6 matches; repeat opponents possible</t>
+          <t>Teams to review</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Small tier: no equally practical, fully assessed split with fewer tiers below 4 teams passes the competitive limits. Review the teams near this break.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>Tier 2 — 3 teams: Double round robin; 4 games each; 6 matches; repeat opponents possible</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>Tiers compare results across whole groups. Teams near a break may still be closely matched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="17" t="inlineStr">
-        <is>
-          <t>Small tier: no equally practical, fully assessed split with fewer tiers below 4 teams passes the competitive limits. Review the teams near this break.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="17" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>Sample data only. Strength markers are observations, not automatic divisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A20:L20"/>
+  <mergeCells count="6">
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A16:L16"/>
-    <mergeCell ref="A19:L19"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A5:L5"/>
     <mergeCell ref="A17:L17"/>
-    <mergeCell ref="A18:L18"/>
-    <mergeCell ref="A3:L3"/>
     <mergeCell ref="A4:L4"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D12">

</xml_diff>

<commit_message>
Refresh MatchBalance teams automatically and simplify director reports (#1345)
* Refresh matched teams automatically and simplify director reports

* Keep refresh available after roster corrections and clarify rollout preflight

* Check refresh controls before Streamlit clears them on rerun
</commit_message>
<xml_diff>
--- a/docs/design/matchbalance-excel/director-workbook-sample.xlsx
+++ b/docs/design/matchbalance-excel/director-workbook-sample.xlsx
@@ -12,9 +12,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'U10 Boys'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$L$18</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'U10 Boys'!$A$1:$L$17</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'U12 Girls'!$1:$6</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$L$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'U12 Girls'!$A$1:$L$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,10 +42,6 @@
     <font>
       <b val="1"/>
       <color rgb="00083E33"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="005B6B66"/>
     </font>
     <font>
       <color rgb="005B6B66"/>
@@ -111,20 +107,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -585,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -616,330 +609,315 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Read from seed 1 down. Tier lines suggest strength divisions; a division can contain several pools. Natural separation marks a strength gap; practical splits also consider usable division sizes. Review warnings and unplaced teams before making final placements.</t>
-        </is>
-      </c>
-    </row>
+    <row r="3" ht="6" customHeight="1"/>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Ratings as of 2026-09-22 · Generated 2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Review-required compromise: 5 teams. Seeded: 5 · Not found in PitchRank: 1 · No current rating: 0 · Data review required: 0</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>5 teams ranked · 1 need placement. Matchup review needed before finalizing</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>MatchBalance seed</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Team name</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Club</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>PowerScore</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>State rank</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>National rank</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Tier / placement</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Final division</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>Pool</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>Final seed</t>
         </is>
       </c>
-      <c r="K6" s="6" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>Director notes</t>
         </is>
       </c>
-      <c r="L6" s="6" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
         <is>
           <t>Record (W-L-D)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Juniper FC 2016 Blue</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Juniper FC</t>
         </is>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="8" t="n">
         <v>90.10000000000001</v>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>AZ #2</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr"/>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="H7" s="11" t="inlineStr"/>
-      <c r="I7" s="11" t="inlineStr"/>
-      <c r="J7" s="12" t="inlineStr"/>
-      <c r="K7" s="11" t="inlineStr"/>
-      <c r="L7" s="7" t="inlineStr"/>
+      <c r="H7" s="10" t="inlineStr"/>
+      <c r="I7" s="10" t="inlineStr"/>
+      <c r="J7" s="11" t="inlineStr"/>
+      <c r="K7" s="10" t="inlineStr"/>
+      <c r="L7" s="6" t="inlineStr"/>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="13" t="n">
+      <c r="A8" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Copper State 2016</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>Copper State</t>
         </is>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="14" t="n">
         <v>87.2</v>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>AZ #6</t>
         </is>
       </c>
-      <c r="F8" s="16" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
+      <c r="F8" s="15" t="inlineStr"/>
+      <c r="G8" s="13" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="H8" s="11" t="inlineStr"/>
-      <c r="I8" s="11" t="inlineStr"/>
-      <c r="J8" s="12" t="inlineStr"/>
-      <c r="K8" s="11" t="inlineStr"/>
-      <c r="L8" s="7" t="inlineStr"/>
+      <c r="H8" s="10" t="inlineStr"/>
+      <c r="I8" s="10" t="inlineStr"/>
+      <c r="J8" s="11" t="inlineStr"/>
+      <c r="K8" s="10" t="inlineStr"/>
+      <c r="L8" s="6" t="inlineStr"/>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Desert United 2016</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Desert United</t>
         </is>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="8" t="n">
         <v>84.59999999999999</v>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>AZ #11</t>
         </is>
       </c>
-      <c r="F9" s="10" t="inlineStr"/>
-      <c r="G9" s="8" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr"/>
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>Tier 1 · Strength gap below</t>
         </is>
       </c>
-      <c r="H9" s="11" t="inlineStr"/>
-      <c r="I9" s="11" t="inlineStr"/>
-      <c r="J9" s="12" t="inlineStr"/>
-      <c r="K9" s="11" t="inlineStr"/>
-      <c r="L9" s="7" t="inlineStr"/>
+      <c r="H9" s="10" t="inlineStr"/>
+      <c r="I9" s="10" t="inlineStr"/>
+      <c r="J9" s="11" t="inlineStr"/>
+      <c r="K9" s="10" t="inlineStr"/>
+      <c r="L9" s="6" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="13" t="n">
+      <c r="A10" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Valley Athletic 2016</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>Valley Athletic</t>
         </is>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="14" t="n">
         <v>72.89999999999999</v>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>AZ #24</t>
         </is>
       </c>
-      <c r="F10" s="16" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
+      <c r="F10" s="15" t="inlineStr"/>
+      <c r="G10" s="13" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="H10" s="11" t="inlineStr"/>
-      <c r="I10" s="11" t="inlineStr"/>
-      <c r="J10" s="12" t="inlineStr"/>
-      <c r="K10" s="11" t="inlineStr"/>
-      <c r="L10" s="7" t="inlineStr"/>
+      <c r="H10" s="10" t="inlineStr"/>
+      <c r="I10" s="10" t="inlineStr"/>
+      <c r="J10" s="11" t="inlineStr"/>
+      <c r="K10" s="10" t="inlineStr"/>
+      <c r="L10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Mesa Juniors 2016</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Mesa Juniors</t>
         </is>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="8" t="n">
         <v>70.09999999999999</v>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>AZ #32</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr"/>
-      <c r="G11" s="8" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr"/>
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="H11" s="11" t="inlineStr"/>
-      <c r="I11" s="11" t="inlineStr"/>
-      <c r="J11" s="12" t="inlineStr"/>
-      <c r="K11" s="11" t="inlineStr"/>
-      <c r="L11" s="7" t="inlineStr"/>
-    </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="13" t="n"/>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="H11" s="10" t="inlineStr"/>
+      <c r="I11" s="10" t="inlineStr"/>
+      <c r="J11" s="11" t="inlineStr"/>
+      <c r="K11" s="10" t="inlineStr"/>
+      <c r="L11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12" ht="15" customHeight="1">
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Sample Academy 2016</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>Sample Academy</t>
         </is>
       </c>
-      <c r="D12" s="13" t="n"/>
-      <c r="E12" s="13" t="inlineStr"/>
-      <c r="F12" s="16" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>Not found in PitchRank · Not found in PitchRank.</t>
-        </is>
-      </c>
-      <c r="H12" s="11" t="inlineStr"/>
-      <c r="I12" s="11" t="inlineStr"/>
-      <c r="J12" s="12" t="inlineStr"/>
-      <c r="K12" s="11" t="inlineStr"/>
-      <c r="L12" s="7" t="inlineStr"/>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="12" t="inlineStr"/>
+      <c r="F12" s="15" t="inlineStr"/>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>Not found in PitchRank.</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr"/>
+      <c r="I12" s="10" t="inlineStr"/>
+      <c r="J12" s="11" t="inlineStr"/>
+      <c r="K12" s="10" t="inlineStr"/>
+      <c r="L12" s="6" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Director notes</t>
+          <t>Teams to review</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="17" t="inlineStr">
-        <is>
-          <t>Tier 1 — 5 teams: Round robin; 4 games each; 10 matches</t>
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Matchup review needed: this split still includes potentially uneven games.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>Matchup review needed: this split still includes potentially uneven games.</t>
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Review this matchup: Juniper FC 2016 Blue vs Mesa Juniors 2016; projected goal gap 4.00, chance of a 4+ goal margin 55%.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>Review this matchup: Juniper FC 2016 Blue vs Mesa Juniors 2016; projected goal gap 4.00, chance of a 4+ goal margin 55%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>Sample workbook: use the yellow columns for the director's final decisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="7">
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A16:L16"/>
     <mergeCell ref="A15:L15"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A5:L5"/>
     <mergeCell ref="A17:L17"/>
-    <mergeCell ref="A18:L18"/>
-    <mergeCell ref="A3:L3"/>
     <mergeCell ref="A4:L4"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D11">
@@ -973,7 +951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1004,379 +982,348 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>Read from seed 1 down. Tier lines suggest strength divisions; a division can contain several pools. Natural separation marks a strength gap; practical splits also consider usable division sizes. Review warnings and unplaced teams before making final placements.</t>
-        </is>
-      </c>
-    </row>
+    <row r="3" ht="6" customHeight="1"/>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Ratings as of 2026-09-22 · Generated 2026-09-25</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Suggested tiers: 3 + 3 teams. Seeded: 6 · Not found in PitchRank: 0 · No current rating: 0 · Data review required: 1</t>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>6 teams ranked · 1 need placement</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>MatchBalance seed</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>Team name</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Club</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>PowerScore</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>State rank</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>National rank</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>Tier / placement</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
+      <c r="H6" s="5" t="inlineStr">
         <is>
           <t>Final division</t>
         </is>
       </c>
-      <c r="I6" s="6" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>Pool</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
         <is>
           <t>Final seed</t>
         </is>
       </c>
-      <c r="K6" s="6" t="inlineStr">
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>Director notes</t>
         </is>
       </c>
-      <c r="L6" s="6" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
         <is>
           <t>Record (W-L-D)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" s="7" t="n">
+      <c r="A7" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Summit SC 2014 Green</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Summit SC</t>
         </is>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="8" t="n">
         <v>89.3</v>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>CO #4</t>
         </is>
       </c>
-      <c r="F7" s="10" t="inlineStr"/>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr"/>
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="H7" s="11" t="inlineStr"/>
-      <c r="I7" s="11" t="inlineStr"/>
-      <c r="J7" s="12" t="inlineStr"/>
-      <c r="K7" s="11" t="inlineStr"/>
-      <c r="L7" s="7" t="inlineStr"/>
+      <c r="H7" s="10" t="inlineStr"/>
+      <c r="I7" s="10" t="inlineStr"/>
+      <c r="J7" s="11" t="inlineStr"/>
+      <c r="K7" s="10" t="inlineStr"/>
+      <c r="L7" s="6" t="inlineStr"/>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="13" t="n">
+      <c r="A8" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Front Range FC 2014</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>Front Range FC</t>
         </is>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="D8" s="14" t="n">
         <v>86.5</v>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>CO #9</t>
         </is>
       </c>
-      <c r="F8" s="16" t="inlineStr"/>
-      <c r="G8" s="14" t="inlineStr">
+      <c r="F8" s="15" t="inlineStr"/>
+      <c r="G8" s="13" t="inlineStr">
         <is>
           <t>Tier 1</t>
         </is>
       </c>
-      <c r="H8" s="11" t="inlineStr"/>
-      <c r="I8" s="11" t="inlineStr"/>
-      <c r="J8" s="12" t="inlineStr"/>
-      <c r="K8" s="11" t="inlineStr"/>
-      <c r="L8" s="7" t="inlineStr"/>
+      <c r="H8" s="10" t="inlineStr"/>
+      <c r="I8" s="10" t="inlineStr"/>
+      <c r="J8" s="11" t="inlineStr"/>
+      <c r="K8" s="10" t="inlineStr"/>
+      <c r="L8" s="6" t="inlineStr"/>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="18" t="n">
+      <c r="A9" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="B9" s="18" t="inlineStr">
         <is>
           <t>Aspen Athletic 2014</t>
         </is>
       </c>
-      <c r="C9" s="19" t="inlineStr">
+      <c r="C9" s="18" t="inlineStr">
         <is>
           <t>Aspen Athletic</t>
         </is>
       </c>
-      <c r="D9" s="20" t="n">
+      <c r="D9" s="19" t="n">
         <v>83.89999999999999</v>
       </c>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>CO #15</t>
         </is>
       </c>
-      <c r="F9" s="21" t="inlineStr"/>
-      <c r="G9" s="19" t="inlineStr">
+      <c r="F9" s="20" t="inlineStr"/>
+      <c r="G9" s="18" t="inlineStr">
         <is>
           <t>Tier 1 · Strength gap below</t>
         </is>
       </c>
-      <c r="H9" s="22" t="inlineStr"/>
-      <c r="I9" s="22" t="inlineStr"/>
-      <c r="J9" s="23" t="inlineStr"/>
-      <c r="K9" s="22" t="inlineStr"/>
-      <c r="L9" s="18" t="inlineStr"/>
+      <c r="H9" s="21" t="inlineStr"/>
+      <c r="I9" s="21" t="inlineStr"/>
+      <c r="J9" s="22" t="inlineStr"/>
+      <c r="K9" s="21" t="inlineStr"/>
+      <c r="L9" s="17" t="inlineStr"/>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="13" t="n">
+      <c r="A10" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Peak United 2014</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>Peak United</t>
         </is>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D10" s="14" t="n">
         <v>71.59999999999999</v>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="E10" s="12" t="inlineStr">
         <is>
           <t>CO #29</t>
         </is>
       </c>
-      <c r="F10" s="16" t="inlineStr"/>
-      <c r="G10" s="14" t="inlineStr">
+      <c r="F10" s="15" t="inlineStr"/>
+      <c r="G10" s="13" t="inlineStr">
         <is>
           <t>Tier 2</t>
         </is>
       </c>
-      <c r="H10" s="11" t="inlineStr"/>
-      <c r="I10" s="11" t="inlineStr"/>
-      <c r="J10" s="12" t="inlineStr"/>
-      <c r="K10" s="11" t="inlineStr"/>
-      <c r="L10" s="7" t="inlineStr"/>
+      <c r="H10" s="10" t="inlineStr"/>
+      <c r="I10" s="10" t="inlineStr"/>
+      <c r="J10" s="11" t="inlineStr"/>
+      <c r="K10" s="10" t="inlineStr"/>
+      <c r="L10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Foothills FC 2014
 Listed: Premier</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Foothills FC</t>
         </is>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="8" t="n">
         <v>68.89999999999999</v>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>CO #37</t>
         </is>
       </c>
-      <c r="F11" s="10" t="inlineStr"/>
-      <c r="G11" s="8" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr"/>
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Tier 2</t>
         </is>
       </c>
-      <c r="H11" s="11" t="inlineStr"/>
-      <c r="I11" s="11" t="inlineStr"/>
-      <c r="J11" s="12" t="inlineStr"/>
-      <c r="K11" s="11" t="inlineStr"/>
-      <c r="L11" s="7" t="inlineStr"/>
+      <c r="H11" s="10" t="inlineStr"/>
+      <c r="I11" s="10" t="inlineStr"/>
+      <c r="J11" s="11" t="inlineStr"/>
+      <c r="K11" s="10" t="inlineStr"/>
+      <c r="L11" s="6" t="inlineStr"/>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="13" t="n">
+      <c r="A12" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Sample Select 2014</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>Sample Select</t>
         </is>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D12" s="14" t="n">
         <v>67.40000000000001</v>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="E12" s="12" t="inlineStr">
         <is>
           <t>CO #42</t>
         </is>
       </c>
-      <c r="F12" s="16" t="inlineStr"/>
-      <c r="G12" s="14" t="inlineStr">
+      <c r="F12" s="15" t="inlineStr"/>
+      <c r="G12" s="13" t="inlineStr">
         <is>
           <t>Tier 2</t>
         </is>
       </c>
-      <c r="H12" s="11" t="inlineStr"/>
-      <c r="I12" s="11" t="inlineStr"/>
-      <c r="J12" s="12" t="inlineStr"/>
-      <c r="K12" s="11" t="inlineStr"/>
-      <c r="L12" s="7" t="inlineStr"/>
+      <c r="H12" s="10" t="inlineStr"/>
+      <c r="I12" s="10" t="inlineStr"/>
+      <c r="J12" s="11" t="inlineStr"/>
+      <c r="K12" s="10" t="inlineStr"/>
+      <c r="L12" s="6" t="inlineStr"/>
     </row>
     <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="7" t="n"/>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Review United 2014</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Review United</t>
         </is>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="8" t="n">
         <v>65</v>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>CO #50</t>
         </is>
       </c>
-      <c r="F13" s="10" t="inlineStr"/>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>Data review required · Confirm the team identity before seeding.</t>
-        </is>
-      </c>
-      <c r="H13" s="11" t="inlineStr"/>
-      <c r="I13" s="11" t="inlineStr"/>
-      <c r="J13" s="12" t="inlineStr"/>
-      <c r="K13" s="11" t="inlineStr"/>
-      <c r="L13" s="7" t="inlineStr"/>
+      <c r="F13" s="9" t="inlineStr"/>
+      <c r="G13" s="7" t="inlineStr">
+        <is>
+          <t>Team data needs review. Confirm the team identity before seeding.</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr"/>
+      <c r="I13" s="10" t="inlineStr"/>
+      <c r="J13" s="11" t="inlineStr"/>
+      <c r="K13" s="10" t="inlineStr"/>
+      <c r="L13" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Director notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>Tier 1 — 3 teams: Double round robin; 4 games each; 6 matches; repeat opponents possible</t>
+          <t>Teams to review</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Small tier: no equally practical, fully assessed split with fewer tiers below 4 teams passes the competitive limits. Review the teams near this break.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>Tier 2 — 3 teams: Double round robin; 4 games each; 6 matches; repeat opponents possible</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>Tiers compare results across whole groups. Teams near a break may still be closely matched.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="30" customHeight="1">
-      <c r="A19" s="17" t="inlineStr">
-        <is>
-          <t>Small tier: no equally practical, fully assessed split with fewer tiers below 4 teams passes the competitive limits. Review the teams near this break.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="17" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>Sample data only. Strength markers are observations, not automatic divisions.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
-    <mergeCell ref="A20:L20"/>
+  <mergeCells count="6">
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A16:L16"/>
-    <mergeCell ref="A19:L19"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A5:L5"/>
     <mergeCell ref="A17:L17"/>
-    <mergeCell ref="A18:L18"/>
-    <mergeCell ref="A3:L3"/>
     <mergeCell ref="A4:L4"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D12">

</xml_diff>